<commit_message>
feat(roles): derive sourced PEM ladder (R3 pilot)
Retrofit Platform Engineering Management to fully-sourced derived rendering
under the cell-derivation/mapping rule: accept OPS-33 (Platform adoption &
deprecation management) into the catalog with a sourced P1-P6 profile, resolve
all 44 competency anchors to bibliography keys (25 new verified sources added),
source every M1-M6 mapping (264 cells) with per-competency why-text checked
against each capability's actual catalog profile rather than pattern-applied,
and harvest the prior authored ladder's role flavor into evidence: lines where
it passes the instance test (264/264 kept). role.yaml is now derived: true;
ladder.md/ladder.csv/ladder.xlsx are mechanically rendered from role.yaml +
catalog, never hand-edited.

check_consistency.py: exit 0, zero REPORT/WARN lines for
platform-engineering-manager. Full test suite: 17 passed.
</commit_message>
<xml_diff>
--- a/roles/platform-engineering-manager/ladder.xlsx
+++ b/roles/platform-engineering-manager/ladder.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Competency Matrix" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Rating Template" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Sources" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Sources &amp; Theory" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -696,20 +696,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K45"/>
+  <dimension ref="A1:L45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="55" customWidth="1" min="7" max="7"/>
     <col width="55" customWidth="1" min="8" max="8"/>
     <col width="55" customWidth="1" min="9" max="9"/>
     <col width="55" customWidth="1" min="10" max="10"/>
     <col width="55" customWidth="1" min="11" max="11"/>
+    <col width="55" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -735,35 +736,40 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Theory Anchor</t>
+          <t>What it covers</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Theory anchor &amp; why</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>M1</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>M2</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>M3</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>M4</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>M5</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>M6</t>
         </is>
@@ -792,37 +798,42 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Schmidt &amp; Hunter, selection-methods meta-analysis (1998)</t>
+          <t>Builds the team through hiring and placement.</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs structured platform-role interview loops against a pre-agreed rubric and work-sample exercise. Defends every hire/no-hire in debrief with recorded signal evidence rather than gut feel. Scope: fills open roles on one platform team.</t>
+          <t>Schmidt &amp; Hunter, The Validity and Utility of Selection Methods in Personnel Psychology, Psychological Bulletin 124(2), 262-274 (1998) — structured, work-sample selection predicts job performance far better than unstructured judgment</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs the loop and rubric for hard-to-fill platform and SRE roles and calibrates interviewers. Rebuilds a loop that is letting weak candidates through by tightening the signals it actually tests. Scope: staffs a critical platform team, senior and specialist hires included.</t>
+          <t>Depth: Shapes hiring for a team; designs loops; makes sound staffing calls. Evidenced by: Defends every hire/no-hire in debrief with recorded signal evidence rather than gut feel. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the hiring bar and interview-design pattern that other platform hiring managers pick up. Publishes the rubric and calibration cadence several teams' loops now run on. Scope: hiring quality across a cross-team platform domain.</t>
+          <t>Depth: Shapes hiring for a team; designs loops; makes sound staffing calls. Evidenced by: Rebuilds a loop that is letting weak candidates through by tightening the signals it actually tests. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the selection system a platform sub-org hires through. Certifies interviewers and installs a bar-raiser mechanism that measurably lifts quality-of-hire. Scope: the hiring pipeline for a platform sub-org.</t>
+          <t>Depth: Drives hiring strategy across teams; builds the interviewing bar. Evidenced by: Publishes the rubric and calibration cadence several teams' loops now run on. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives the function's talent strategy, weighing grow-vs-buy for scarce reliability and DevEx skills. Shapes leveling and headcount decisions across the function from pipeline and labor-market data. Scope: the platform function's talent supply.</t>
+          <t>Depth: Drives hiring strategy across teams; builds the interviewing bar. Evidenced by: Certifies interviewers and installs a bar-raiser mechanism that measurably lifts quality-of-hire. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide philosophy for hiring platform and infrastructure talent that peer functions benchmark against. Pioneers selection practice, like work-sample design for platform work, that other organizations copy. Scope: company-wide platform talent bar and brand.</t>
+          <t>Depth: Sets the org's talent strategy. Evidenced by: Shapes leveling and headcount decisions across the function from pipeline and labor-market data. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Shapes company-wide talent philosophy. Evidenced by: Pioneers selection practice, like work-sample design for platform work, that other organizations copy. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -849,37 +860,42 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Tuckman, Developmental Sequence in Small Groups (1965)</t>
+          <t>Ramps new people to productivity fast and leads teams through formation stages — launches, merges, and resets — deliberately rather than enduring them.</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs a structured onboarding with a buddy, a ramp checklist, and a first paved-road change in week one. Gets a new platform hire shipping a real change within their first sprint. Scope: onboarding into one platform team.</t>
+          <t>Tuckman, Developmental Sequence in Small Groups, Psychological Bulletin 63(6), 384-399 (1965) — teams cross forming-storming-norming-performing, and the manager's job is to shorten that arc</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs onboarding for a high-stakes team where on-call and blast radius are real, sequencing access, shadowing, and first incident exposure. Reads where a forming team is stuck in storming and intervenes to move it to performing. Scope: team formation on a critical platform team.</t>
+          <t>Depth: Runs a 30/60/90 onboarding with named buddies and early wins; new hires ship in their first weeks and say so in check-ins. Evidenced by: Gets a new platform hire shipping a real change within their first sprint. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the onboarding and team-formation standard other platform leads adopt. Ships a reusable ramp template and 30/60/90 model that cuts time-to-first-contribution across the domain. Scope: onboarding quality across a cross-team platform domain.</t>
+          <t>Depth: Reads a team's formation stage and intervenes on it — resets norms after a merge, names storming in the room instead of managing it by email. Evidenced by: Reads where a forming team is stuck in storming and intervenes to move it to performing. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the operating rhythm that forms and re-forms teams cleanly through platform re-splits across a sub-org. Stands up a new platform team from scratch to productive without a delivery trough. Scope: team formation across a platform sub-org.</t>
+          <t>Depth: Builds the onboarding and team-launch playbook multiple teams use; teams start faster because of materials and rituals they created, and stands up whole new teams repeatedly. Evidenced by: Ships a reusable ramp template and 30/60/90 model that cuts time-to-first-contribution across the domain. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives how the function grows, splits, and merges teams as demand shifts while keeping Team-Topologies boundaries clean. Sets the norms that keep newly formed platform teams productive through function-wide scaling. Scope: team formation across the platform function.</t>
+          <t>Depth: Builds the onboarding and team-launch playbook multiple teams use; teams start faster because of materials and rituals they created, and stands up whole new teams repeatedly. Evidenced by: Stands up a new platform team from scratch to productive without a delivery trough. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide model for how platform capability is stood up and dissolved as bets change. Pioneers the team-formation playbook other engineering functions reuse. Scope: org-wide platform team topology.</t>
+          <t>Depth: Designs how an organization absorbs step-change growth — acquisitions, new sites, doubled headcount — without culture dilution; integration plans carry named cultural mechanisms. Evidenced by: Sets the norms that keep newly formed platform teams productive through function-wide scaling. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Makes team formation an organization-wide capability — new groups spin up predictably without heroics — and audits that the machinery still works. Evidenced by: Pioneers the team-formation playbook other engineering functions reuse. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -906,37 +922,42 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Whitmore, Coaching for Performance (1992); Google Project Oxygen</t>
+          <t>Grows other people's capability.</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Depth: Holds regular 1:1s that coach rather than status-check, favoring questions over answers. Turns a specific platform-engineer weakness into a visible skill gain within a quarter. Scope: coaches the engineers on one platform team.</t>
+          <t>Whitmore, Coaching for Performance: GROWing Human Potential and Purpose, 4th ed. (Nicholas Brealey, 2009; orig. 1992) — regular coaching, not status-checking, is the top driver of manager effectiveness</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Depth: Coaches senior engineers and tech leads through ambiguous, high-judgment work such as reliability trade-offs and on-call leadership. Develops a report into a tech lead who now runs a workstream unaided. Scope: develops the talent bench of a critical platform team.</t>
+          <t>Depth: Coaches engineers with growth-oriented feedback; measurably improves a team's skill. Evidenced by: Turns a specific platform-engineer weakness into a visible skill gain within a quarter. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Depth: Grows other people-leaders' coaching skill, not just individuals'. Runs coaching-the-coach sessions that lift how platform leads across the domain develop their own people. Scope: coaching capability across a cross-team platform domain.</t>
+          <t>Depth: Coaches engineers with growth-oriented feedback; measurably improves a team's skill. Evidenced by: Develops a report into a tech lead who now runs a workstream unaided. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the leadership-development pipeline a platform sub-org relies on, growing future platform leaders before seats open. Produces leaders others actively recruit onto their teams. Scope: the leadership bench of a platform sub-org.</t>
+          <t>Depth: Develops future leads across teams; shapes hiring and onboarding. Evidenced by: Runs coaching-the-coach sessions that lift how platform leads across the domain develop their own people. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives the function's approach to growing engineering and management talent, tied to the reliability and DevEx skills it will need. Sets development standards leaders across the function coach against. Scope: talent development across the platform function.</t>
+          <t>Depth: Develops future leads across teams; shapes hiring and onboarding. Evidenced by: Produces leaders others actively recruit onto their teams. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide expectation for how platform leaders are grown. Pioneers a development model peer functions adopt. Scope: company-wide platform leadership development.</t>
+          <t>Depth: Develops senior engineers and leaders; builds culture deliberately. Evidenced by: Sets development standards leaders across the function coach against. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Develops the next generation of top talent; legacy outlasts tenure. Evidenced by: Pioneers a development model peer functions adopt. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -963,37 +984,42 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Hewlett, Forget a Mentor, Find a Sponsor (2013)</t>
+          <t>Growing engineers through development plans, advancement opportunities, and active sponsorship.</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Depth: Holds career conversations and writes growth plans tied to the ladder. Puts a report's name forward for a visible platform project that stretches them. Scope: career growth for one platform team.</t>
+          <t>Hewlett, Forget a Mentor, Find a Sponsor: The New Way to Fast-Track Your Career (Harvard Business Review Press, 2013) — advancement comes from spending capital on people, not just mentoring them</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sponsors senior engineers into stretch scope and promotion, building the evidence case ahead of calibration. Gets a deserving platform engineer promoted through a defensible packet. Scope: advancement on a critical platform team.</t>
+          <t>Depth: Coaches direct reports on standard career growth with normal review. Evidenced by: Puts a report's name forward for a visible platform project that stretches them. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets sponsorship norms other platform leads adopt. Advocates for talent in cross-team calibration rooms they do not own, moving outcomes for people who are not theirs. Scope: advancement across a cross-team platform domain.</t>
+          <t>Depth: Independently sponsors people into stretch roles and navigates complex growth paths. Evidenced by: Gets a deserving platform engineer promoted through a defensible packet. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the succession and sponsorship system for a platform sub-org so key roles have ready successors. Spends visible capital to place emerging platform leaders into scope. Scope: succession across a platform sub-org.</t>
+          <t>Depth: Defines career-development practices others adopt and unblocks the toughest growth cases. Evidenced by: Advocates for talent in cross-team calibration rooms they do not own, moving outcomes for people who are not theirs. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives the function's approach to advancing and retaining top talent, including the scarce staff-plus platform-architect and reliability track. Sets the sponsorship expectations leaders across the function are held to. Scope: advancement across the platform function.</t>
+          <t>Depth: Defines career-development practices others adopt and unblocks the toughest growth cases. Evidenced by: Spends visible capital to place emerging platform leaders into scope. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide standard for how platform careers ladder. Pioneers a sponsorship model that measurably widens the platform leadership pipeline. Scope: company-wide platform career paths.</t>
+          <t>Depth: Sets the org's talent-development strategy and anticipates future capability needs. Evidenced by: Sets the sponsorship expectations leaders across the function are held to. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines exemplary career sponsorship for the discipline and is externally recognized for it. Evidenced by: Pioneers a sponsorship model that measurably widens the platform leadership pipeline. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -1020,37 +1046,42 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Grove, High Output Management (1983)</t>
+          <t>Setting expectations, evaluating performance, and addressing under-performance fairly and clearly.</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets clear expectations and gives specific, timely feedback. Addresses an underperforming platform engineer directly with a documented plan rather than letting it drift. Scope: performance on one platform team.</t>
+          <t>Grove, High Output Management (Random House, 1983) — a manager's output is the team's output, so managing performance is the core lever</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Depth: Manages the full performance range on a high-stakes team, rewarding top reliability contributors and fairly turning around or exiting persistent underperformance. Runs a difficult exit cleanly and defensibly. Scope: performance on a critical platform team.</t>
+          <t>Depth: Independently manages underperformance and difficult cases through to clear resolution. Evidenced by: Addresses an underperforming platform engineer directly with a documented plan rather than letting it drift. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the performance and calibration standard other platform leads apply consistently. Runs cross-team calibration that holds a fair, comparable bar across the domain. Scope: performance consistency across a cross-team platform domain.</t>
+          <t>Depth: Independently manages underperformance and difficult cases through to clear resolution. Evidenced by: Runs a difficult exit cleanly and defensibly. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the performance system a platform sub-org runs on, from level expectations to calibration mechanics. Corrects rating drift between teams so the bar means the same everywhere. Scope: performance management across a platform sub-org.</t>
+          <t>Depth: Defines accountability practices other managers adopt and coaches them through hard cases. Evidenced by: Runs cross-team calibration that holds a fair, comparable bar across the domain. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives the function's performance philosophy and its link to reliability and delivery outcomes. Sets the standard leaders across the function calibrate to. Scope: performance across the platform function.</t>
+          <t>Depth: Defines accountability practices other managers adopt and coaches them through hard cases. Evidenced by: Corrects rating drift between teams so the bar means the same everywhere. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide performance expectations for platform leadership. Pioneers a performance model peer functions adopt. Scope: company-wide platform performance standard.</t>
+          <t>Depth: Sets the org's performance philosophy and anticipates systemic accountability gaps. Evidenced by: Sets the standard leaders across the function calibrate to. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines what fair, effective performance management means and influences the field externally. Evidenced by: Pioneers a performance model peer functions adopt. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -1077,37 +1108,42 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Edmondson, The Fearless Organization (2018); Project Aristotle</t>
+          <t>Creates the conditions where people raise problems, dissent, and admit mistakes without penalty; reads and repairs team-health signals (conflict, burnout risk, on-call load).</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs blameless retros and incident reviews and invites dissent. Models admitting their own mistakes so engineers surface problems early instead of hiding them. Scope: team health on one platform team.</t>
+          <t>Edmondson, The Fearless Organization: Creating Psychological Safety in the Workplace for Learning, Innovation, and Growth (Wiley, 2018) — safety is the top predictor of team performance and the precondition for blameless ops</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sustains safety on a high-pressure on-call team where incidents are public and stressful. Keeps a severe-outage review blameless so the real contributing causes come out. Scope: team health on a critical platform team.</t>
+          <t>Depth: Sustains safety through pressure (incidents, deadlines, change); repairs damaged trust; the team measurably speaks up (postmortems name real causes). Evidenced by: Models admitting their own mistakes so engineers surface problems early instead of hiding them. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the team-health and blameless-culture standard other platform leads adopt. Instruments team-health signals across the domain and acts on a declining one before it becomes attrition. Scope: team health across a cross-team platform domain.</t>
+          <t>Depth: Sustains safety through pressure (incidents, deadlines, change); repairs damaged trust; the team measurably speaks up (postmortems name real causes). Evidenced by: Keeps a severe-outage review blameless so the real contributing causes come out. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the culture mechanisms a platform sub-org relies on, from survey cadence to blameless-review norms and safety expectations for leaders. Turns around an unhealthy team's culture through the leader running it. Scope: culture across a platform sub-org.</t>
+          <t>Depth: Diagnoses and fixes systemic safety failures across teams; other leaders seek their help on entrenched conflict and burnout patterns. Evidenced by: Instruments team-health signals across the domain and acts on a declining one before it becomes attrition. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives the function's culture, tying psychological safety explicitly to reliability outcomes. Sets the health norms leaders across the function are measured against. Scope: culture across the platform function.</t>
+          <t>Depth: Diagnoses and fixes systemic safety failures across teams; other leaders seek their help on entrenched conflict and burnout patterns. Evidenced by: Turns around an unhealthy team's culture through the leader running it. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide expectation that platform operates blamelessly and safely. Pioneers a culture model other engineering functions copy. Scope: company-wide platform culture.</t>
+          <t>Depth: Sets the org's team-health bar and mechanisms; safety practices they designed are adopted org-wide. Evidenced by: Sets the health norms leaders across the function are measured against. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Shapes how the industry thinks about team health; published practices others implement. Evidenced by: Pioneers a culture model other engineering functions copy. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -1134,37 +1170,42 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Deci &amp; Ryan, Self-Determination Theory (2000); Herzberg (1968)</t>
+          <t>Builds durable intrinsic motivation: removes dissatisfiers, feeds autonomy/mastery/purpose, recognizes well.</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Depth: Reads what motivates each engineer and connects platform work to purpose. Spots a disengaging report early and re-engages them before they start looking. Scope: engagement on one platform team.</t>
+          <t>Deci &amp; Ryan, The "What" and "Why" of Goal Pursuits: Human Needs and the Self-Determination of Behavior, Psychological Inquiry 11(4), 227-268 (2000) — autonomy, mastery, and purpose drive durable engagement more than extrinsic rewards</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sustains engagement on a team doing high-toil, sometimes thankless reliability work by framing impact and rotating growth. Keeps regrettable attrition low on a critical platform team through a demanding period. Scope: retention on a critical platform team.</t>
+          <t>Depth: Sustains engagement through hard stretches; diagnoses systemic motivation problems (not just individuals) and fixes the conditions. Evidenced by: Spots a disengaging report early and re-engages them before they start looking. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets engagement and retention practices other platform leads adopt. Reads engagement signals across the domain and fixes a systemic driver of attrition, not just symptoms. Scope: engagement across a cross-team platform domain.</t>
+          <t>Depth: Sustains engagement through hard stretches; diagnoses systemic motivation problems (not just individuals) and fixes the conditions. Evidenced by: Keeps regrettable attrition low on a critical platform team through a demanding period. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the retention strategy a platform sub-org runs on, targeting the drivers specific to platform work such as toil, on-call load, and low visibility. Shifts a sub-org's engagement trend through the leaders who own each team. Scope: retention across a platform sub-org.</t>
+          <t>Depth: Builds engagement mechanisms other teams adopt; reverses disengagement trends beyond their own span. Evidenced by: Reads engagement signals across the domain and fixes a systemic driver of attrition, not just symptoms. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives the function's engagement and retention strategy, protecting scarce reliability and DevEx talent. Sets the expectations leaders across the function own for engagement. Scope: retention across the platform function.</t>
+          <t>Depth: Builds engagement mechanisms other teams adopt; reverses disengagement trends beyond their own span. Evidenced by: Shifts a sub-org's engagement trend through the leaders who own each team. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide narrative that makes platform a destination rather than a cost center. Pioneers retention practice for infrastructure talent that peers adopt. Scope: company-wide platform engagement.</t>
+          <t>Depth: Owns the engagement strategy for a function; conditions they designed show up in retention and survey trends. Evidenced by: Sets the expectations leaders across the function own for engagement. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Advances the practice of engagement in the field; frameworks others cite and use. Evidenced by: Pioneers retention practice for infrastructure talent that peers adopt. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -1191,37 +1232,42 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Perri, Escaping the Build Trap (2018); Skelton &amp; Pais, Team Topologies (2019)</t>
+          <t>Sequencing initiatives across products and horizons against goals, capacity, and dependencies.</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Depth: Maintains a platform roadmap tied to developer outcomes, not just a feature list. States the problem each platform capability solves and for whom. Scope: the roadmap for one platform team's surface.</t>
+          <t>Perri, Escaping the Build Trap: How Effective Product Management Creates Real Value (O'Reilly, 2018) — a platform is run as a product with outcomes and sized as a thinnest-viable-platform, not a feature factory</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Depth: Owns the vision and roadmap for a critical platform area, sequencing by developer value and thinnest-viable-platform thinking. Kills or defers a low-value platform build others wanted, with the outcome argument to back it. Scope: roadmap for a high-stakes platform team.</t>
+          <t>Depth: Builds and sequences a credible roadmap for one product with normal review. Evidenced by: States the problem each platform capability solves and for whom. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets a cross-team platform vision that other teams' roadmaps align to. Publishes a domain platform strategy that redirects several teams' build priorities. Scope: platform direction across a cross-team domain.</t>
+          <t>Depth: Independently balances competing priorities and replans confidently under shifting constraints. Evidenced by: Kills or defers a low-value platform build others wanted, with the outcome argument to back it. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the multi-year platform roadmap a sub-org executes against, balancing capability bets, migrations, and retirement. Frames the platform-as-a-product operating model the sub-org plans within. Scope: platform strategy for a sub-org.</t>
+          <t>Depth: Designs the planning approach others use and resolves cross-team portfolio conflicts. Evidenced by: Publishes a domain platform strategy that redirects several teams' build priorities. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives the function's vision and its link to business outcomes and developer productivity. Sets the platform bets the function organizes around and defends them at the exec table. Scope: vision for the platform function.</t>
+          <t>Depth: Designs the planning approach others use and resolves cross-team portfolio conflicts. Evidenced by: Frames the platform-as-a-product operating model the sub-org plans within. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide platform vision and the make-vs-consume posture for the whole company. Pioneers a platform strategy the industry recognizes. Scope: org-wide platform direction.</t>
+          <t>Depth: Sets portfolio planning strategy and foresees where investment should shift next. Evidenced by: Sets the platform bets the function organizes around and defends them at the exec table. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines portfolio-planning best practice for the field and is recognized for it. Evidenced by: Pioneers a platform strategy the industry recognizes. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -1248,37 +1294,42 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Noda, Storey, Forsgren &amp; Greiler, DevEx: What Actually Drives Productivity (ACM Queue, 2023)</t>
+          <t>Uncovering user needs and validating problems through interviews, observation, and experimentation.</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Depth: Talks to platform users regularly and watches them use the tools. Turns an observed developer pain point into a prioritized platform fix. Scope: discovery for one platform team's users.</t>
+          <t>Noda, Storey, Forsgren &amp; Greiler, DevEx: What Actually Drives Productivity, ACM Queue 21(2) (2023) — platform value is set by developers' lived experience, which must be measured not assumed</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs structured DevEx discovery for a critical platform area through interviews, journey mapping, and friction logs. Quantifies a cognitive-load or feedback-loop problem the team then designs against. Scope: discovery for a high-stakes platform team's users.</t>
+          <t>Depth: Plans and conducts standard discovery for a feature, synthesizing themes with normal review. Evidenced by: Turns an observed developer pain point into a prioritized platform fix. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the DevEx-research practice other platform teams adopt. Stands up a developer-experience measurement combining surveys and system signals that several teams now steer by. Scope: DevEx discovery across a cross-team domain.</t>
+          <t>Depth: Independently frames ambiguous problems, selects fitting methods, and separates signal from noise. Evidenced by: Quantifies a cognitive-load or feedback-loop problem the team then designs against. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the continuous developer-listening system a platform sub-org runs on, linking perceptual and system metrics. Makes DevEx evidence the default input to roadmap decisions across the sub-org. Scope: developer research across a platform sub-org.</t>
+          <t>Depth: Designs the team's discovery approach and untangles findings others find contradictory. Evidenced by: Stands up a developer-experience measurement combining surveys and system signals that several teams now steer by. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives how the function understands and represents developer productivity to the business. Sets the DevEx metrics the function commits to and reports upward. Scope: developer insight across the platform function.</t>
+          <t>Depth: Designs the team's discovery approach and untangles findings others find contradictory. Evidenced by: Makes DevEx evidence the default input to roadmap decisions across the sub-org. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide definition of developer experience and how it is measured. Pioneers a DevEx research program other companies reference. Scope: org-wide developer-experience insight.</t>
+          <t>Depth: Sets the org's research strategy and anticipates emerging customer needs before they surface. Evidenced by: Sets the DevEx metrics the function commits to and reports upward. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines what rigorous product discovery means and shapes the discipline's practice externally. Evidenced by: Pioneers a DevEx research program other companies reference. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -1305,37 +1356,42 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Cagan, Inspired (2008)</t>
+          <t>Connects technical work to user and business value.</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Depth: Articulates the value of the team's platform work in developer-time and reliability terms. Ties a platform initiative to a concrete productivity or cost outcome. Scope: value case for one platform team.</t>
+          <t>Cagan, INSPIRED: How to Create Tech Products Customers Love, 2nd Edition (Wiley, 2018) — platform investment is justified in value delivered, not output shipped</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the business case for a significant platform investment, quantifying time saved, incidents avoided, or spend reduced. Wins funding for a platform bet with a defensible value model. Scope: value case for a critical platform team's investments.</t>
+          <t>Depth: Frames own work in user/business outcomes, not just tasks. Evidenced by: Ties a platform initiative to a concrete productivity or cost outcome. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the value-articulation standard other platform leads use. Publishes a value and ROI framework several teams justify platform work with. Scope: platform value cases across a cross-team domain.</t>
+          <t>Depth: Treats their area as a product; uses metrics to decide what to build for a domain. Evidenced by: Wins funding for a platform bet with a defensible value model. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the investment model a platform sub-org allocates by, ranking bets on value and leverage. Reframes platform from cost center to leverage multiplier for the sub-org's stakeholders. Scope: investment cases across a platform sub-org.</t>
+          <t>Depth: Expert at aligning technical bets with product strategy across teams. Evidenced by: Publishes a value and ROI framework several teams justify platform work with. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives how the function proves and communicates its business value. Sets the value narrative and metrics the function is funded against. Scope: value case for the platform function.</t>
+          <t>Depth: Expert at aligning technical bets with product strategy across teams. Evidenced by: Reframes platform from cost center to leverage multiplier for the sub-org's stakeholders. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide economic case for platform investment. Pioneers a platform-value model the business plans capital around. Scope: org-wide platform economics.</t>
+          <t>Depth: Sets product direction for an org's technical surface. Evidenced by: Sets the value narrative and metrics the function is funded against. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Shapes how the company creates value through technical products. Evidenced by: Pioneers a platform-value model the business plans capital around. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -1362,37 +1418,42 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Spotify Engineering, How We Use Golden Paths (2020)</t>
+          <t>Build self-service internal platforms and paved paths that streamline delivery.</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Depth: Maintains a golden path for a common workflow that is templated, documented, and supported. Gets the team's users onto the paved road for one high-frequency task. Scope: golden paths on one platform team's surface.</t>
+          <t>Spotify Engineering, How We Use Golden Paths to Solve Fragmentation in Our Software Ecosystem (Spotify Engineering Blog, 2020) — an opinionated, supported path makes the right way the easy way</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs paved roads for a critical platform area, balancing opinion with escape hatches. Retires a fragmented set of bespoke setups onto a single supported golden path. Scope: paved roads for a high-stakes platform team.</t>
+          <t>Depth: Independently builds and supports standard platform capabilities and templates for routine developer needs with review. Evidenced by: Gets the team's users onto the paved road for one high-frequency task. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the golden-path design standard other platform teams adopt. Defines what paved means across the domain, from support SLA to versioning and deprecation, and gets teams to build to it. Scope: paved-road strategy across a cross-team domain.</t>
+          <t>Depth: Designs self-service workflows for ambiguous needs, reducing friction and resolving hard abstraction and adoption issues. Evidenced by: Retires a fragmented set of bespoke setups onto a single supported golden path. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the paved-road portfolio a platform sub-org offers and the governance that keeps it coherent. Makes the golden path the default choice across the sub-org, not the exception. Scope: paved roads across a platform sub-org.</t>
+          <t>Depth: Defines platform architecture and golden paths others adopt, solving deep developer-experience and leverage problems. Evidenced by: Defines what paved means across the domain, from support SLA to versioning and deprecation, and gets teams to build to it. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives the function's golden-path strategy and the trade-off between standardization and team autonomy. Sets the paved-road principles the whole function designs to. Scope: paved-road direction across the platform function.</t>
+          <t>Depth: Defines platform architecture and golden paths others adopt, solving deep developer-experience and leverage problems. Evidenced by: Makes the golden path the default choice across the sub-org, not the exception. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide philosophy of paved roads versus freedom. Pioneers a golden-path model other engineering orgs adopt. Scope: org-wide paved-road strategy.</t>
+          <t>Depth: Sets organization-wide platform strategy, anticipating how developer-experience engineering should evolve. Evidenced by: Sets the paved-road principles the whole function designs to. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines what excellent platform engineering means for the field, shaping industry developer-experience practice. Evidenced by: Pioneers a golden-path model other engineering orgs adopt. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -1419,37 +1480,42 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Bottcher, What I Talk About When I Talk About Platforms (martinfowler.com, 2018)</t>
+          <t>Build self-service internal platforms and paved paths that streamline delivery.</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Depth: Keeps a self-service interface such as a portal, CLI, API, or template working for a common request so users do not file tickets. Eliminates a manual request path by making it self-serve. Scope: self-service on one platform team's surface.</t>
+          <t>Bottcher, What I Talk About When I Talk About Platforms (martinfowler.com, 2018) — a platform's job is to cut cognitive load through interfaces developers use without asking anyone</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs self-service for a critical platform capability with the right abstraction level and guardrails. Removes the team as a human bottleneck from a high-volume workflow. Scope: self-service for a high-stakes platform team.</t>
+          <t>Depth: Independently builds and supports standard platform capabilities and templates for routine developer needs with review. Evidenced by: Eliminates a manual request path by making it self-serve. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the self-service and interface standard other teams adopt. Defines the interface-contract pattern, whether API, portal, or paved road, that several platform teams now expose. Scope: self-service design across a cross-team domain.</t>
+          <t>Depth: Designs self-service workflows for ambiguous needs, reducing friction and resolving hard abstraction and adoption issues. Evidenced by: Removes the team as a human bottleneck from a high-volume workflow. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the self-service platform model a sub-org runs on, a coherent developer surface rather than scattered tools. Shifts the sub-org's platforms from ticket-driven to self-service by default. Scope: platform interfaces across a platform sub-org.</t>
+          <t>Depth: Defines platform architecture and golden paths others adopt, solving deep developer-experience and leverage problems. Evidenced by: Defines the interface-contract pattern, whether API, portal, or paved road, that several platform teams now expose. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives the function's self-service strategy and its internal-developer-platform vision. Sets the target that platform work is consumed without human intervention across the function. Scope: self-service direction across the platform function.</t>
+          <t>Depth: Defines platform architecture and golden paths others adopt, solving deep developer-experience and leverage problems. Evidenced by: Shifts the sub-org's platforms from ticket-driven to self-service by default. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide bar for developer self-service. Pioneers an internal-platform interface model the industry references. Scope: org-wide self-service platform.</t>
+          <t>Depth: Sets organization-wide platform strategy, anticipating how developer-experience engineering should evolve. Evidenced by: Sets the target that platform work is consumed without human intervention across the function. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines what excellent platform engineering means for the field, shaping industry developer-experience practice. Evidenced by: Pioneers an internal-platform interface model the industry references. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -1471,42 +1537,47 @@
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>OPS-33</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Winters, Manshreck &amp; Wright, Software Engineering at Google (2020) - deprecation chapter</t>
+          <t>Drives internal adoption of platform capabilities and manages the full lifecycle of platform surfaces - migration onto paved roads, long-tail burndown, and safe deprecation and sunsetting of what they replace.</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives adoption of a platform capability by making migration easy with codemods, docs, and hands-on help. Moves the first cohort of teams onto a new platform version. Scope: adoption on one platform team's surface.</t>
+          <t>Winters, Manshreck &amp; Wright, Software Engineering at Google: Lessons Learned from Programming Over Time (O'Reilly, 2020) — a platform only creates value once adopted, and migrations and deprecations must be engineered and finished, not merely mandated</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs a migration for a critical platform area, tracking adoption and burning down the long tail. Completes a migration including the last stubborn holdouts rather than stalling at eighty percent. Scope: migration for a high-stakes platform capability.</t>
+          <t>Depth: Runs the adoption of a single capability end to end - communicates the change, provides migration tooling or docs, and clears the common blockers without help. Evidenced by: Moves the first cohort of teams onto a new platform version. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the adoption and deprecation strategy other platform teams follow. Defines the deprecation policy and migration-support standard several teams' rollouts now run on. Scope: adoption strategy across a cross-team domain.</t>
+          <t>Depth: Owns a capability's adoption and deprecation as a program: sets migration tooling (codemods, automated rewrites), burns down the long tail, and enforces a deprecation policy with published timelines and support commitments. Evidenced by: Completes a migration including the last stubborn holdouts rather than stalling at eighty percent. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the migration operating model a sub-org uses, with incentives, tracking, and deprecation guarantees so platform change lands without stranding teams. Drives a sub-org-wide migration to completion through the teams that own each service. Scope: migration across a platform sub-org.</t>
+          <t>Depth: Designs the migration operating model a domain reuses - adoption instrumentation, incentives, and deprecation guarantees - so multiple teams retire and replace surfaces predictably. Evidenced by: Defines the deprecation policy and migration-support standard several teams' rollouts now run on. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives the function's adoption strategy and its balance of carrots versus mandates. Sets the adoption and sunsetting principles the function commits to. Scope: adoption direction across the platform function.</t>
+          <t>Depth: Designs the migration operating model a domain reuses - adoption instrumentation, incentives, and deprecation guarantees - so multiple teams retire and replace surfaces predictably. Evidenced by: Drives a sub-org-wide migration to completion through the teams that own each service. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide expectation for how platforms are adopted and legacy is retired. Pioneers a migration model that keeps the org off long-lived forks. Scope: org-wide adoption and deprecation.</t>
+          <t>Depth: Sets the organization's adoption and deprecation standards: the sunset principles, the guarantee bar, and the mechanisms that keep the platform's surface area from sprawling as it grows. Evidenced by: Sets the adoption and sunsetting principles the function commits to. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Establishes adoption-and-lifecycle practice others in the field adopt; makes deprecation a trusted, low-friction default rather than a feared event across the industry. Evidenced by: Pioneers a migration model that keeps the org off long-lived forks. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -1533,37 +1604,42 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>CNCF TAG App Delivery, Platform Engineering Maturity Model (2023)</t>
+          <t>Growing and nurturing developer communities and representing their needs internally.</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs enablement for the platform through docs, office hours, and demos. Turns a confused user base into a competent one for one capability through documentation and support. Scope: advocacy for one platform team's users.</t>
+          <t>CNCF TAG App Delivery, Platform Engineering Maturity Model (2023) — platforms succeed on enablement and advocacy as much as on the technology</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the enablement program for a critical platform area, from onboarding guides to champions and feedback channels. Grows an internal champion network that advocates the platform without the team present. Scope: enablement for a high-stakes platform team.</t>
+          <t>Depth: Grows and supports a developer community segment with normal review. Evidenced by: Turns a confused user base into a competent one for one capability through documentation and support. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the advocacy and enablement standard other platform teams adopt. Stands up a platform-community and docs practice several teams run their enablement through. Scope: enablement across a cross-team domain.</t>
+          <t>Depth: Independently builds thriving communities and defuses tense community conflicts. Evidenced by: Grows an internal champion network that advocates the platform without the team present. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the developer-relations model a platform sub-org uses to drive internal awareness and adoption. Makes platform enablement a repeatable function rather than heroics across the sub-org. Scope: advocacy across a platform sub-org.</t>
+          <t>Depth: Defines community-building practices others adopt and revives flagging communities. Evidenced by: Stands up a platform-community and docs practice several teams run their enablement through. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives how the function positions and evangelizes itself to engineering and the business. Sets the enablement and advocacy strategy the function invests in. Scope: advocacy across the platform function.</t>
+          <t>Depth: Defines community-building practices others adopt and revives flagging communities. Evidenced by: Makes platform enablement a repeatable function rather than heroics across the sub-org. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide platform-advocacy posture. Pioneers an internal developer-relations model peer functions and other orgs copy. Scope: org-wide platform advocacy.</t>
+          <t>Depth: Sets the org's community strategy and anticipates where developer interest is shifting. Evidenced by: Sets the enablement and advocacy strategy the function invests in. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines what great developer advocacy means and is externally recognized for it. Evidenced by: Pioneers an internal developer-relations model peer functions and other orgs copy. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -1590,37 +1666,42 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Beyer, Jones, Petoff &amp; Murphy, Site Reliability Engineering (2016)</t>
+          <t>Keeps services healthy; designs for failure.</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs the team's services on defined SLOs and error budgets and reviews budget burn. Uses an error-budget breach to hold a release-versus-reliability trade-off honestly. Scope: SLOs for one platform team's services.</t>
+          <t>Beyer, Jones, Petoff &amp; Murphy (eds.), Site Reliability Engineering: How Google Runs Production Systems (O'Reilly/Google, 2016) — SLOs and error budgets turn reliability from opinion into an explicit, negotiable target</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs the SLO and error-budget model for a critical platform area with meaningful SLIs. Negotiates and enforces an error-budget policy that pauses feature work when reliability slips. Scope: reliability targets for a high-stakes platform team.</t>
+          <t>Depth: Builds retries, timeouts and fallbacks; understands blast radius. Evidenced by: Uses an error-budget breach to hold a release-versus-reliability trade-off honestly. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the SLO and error-budget standard other platform teams adopt. Defines the reliability-target framework several teams now run their services against. Scope: reliability targets across a cross-team domain.</t>
+          <t>Depth: Designs for graceful degradation; defines SLOs; accountable for a domain's reliability. Evidenced by: Negotiates and enforces an error-budget policy that pauses feature work when reliability slips. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the reliability operating model a sub-org runs on, from SLO taxonomy to budget governance and reliability reviews. Makes error-budget policy the mechanism the sub-org's prioritization respects. Scope: reliability across a platform sub-org.</t>
+          <t>Depth: Expert in resilience and capacity planning at scale; drives down incidents systemically. Evidenced by: Defines the reliability-target framework several teams now run their services against. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives the function's reliability strategy and its explicit trade-off with velocity. Sets the reliability commitments the function makes to the business. Scope: reliability across the platform function.</t>
+          <t>Depth: Expert in resilience and capacity planning at scale; drives down incidents systemically. Evidenced by: Makes error-budget policy the mechanism the sub-org's prioritization respects. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide reliability philosophy and the availability posture the company commits to customers. Pioneers a reliability model other orgs adopt. Scope: org-wide reliability.</t>
+          <t>Depth: Owns org-level reliability; fixes risk in process and org design. Evidenced by: Sets the reliability commitments the function makes to the business. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Sets the company's reliability philosophy. Evidenced by: Pioneers a reliability model other orgs adopt. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -1647,37 +1728,42 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>PagerDuty, Incident Response Guide (2017); Allspaw, Blameless PostMortems (2012)</t>
+          <t>Establishing on-call, incident response, and risk practices that protect reliability.</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs the team's on-call and incident process and acts as commander when needed. Turns a postmortem's action items into shipped fixes rather than a filed document. Scope: incident response on one platform team.</t>
+          <t>PagerDuty, Incident Response Documentation (accessed 2026-07) — how an org runs incidents and blameless learning decides whether outages recur</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Depth: Leads response for severe, cross-team incidents on a critical platform, coordinating comms and command under pressure. Runs a major-incident review whose systemic fixes prevent the class of failure from recurring. Scope: incident leadership for a high-stakes platform.</t>
+          <t>Depth: Manages standard incidents and routine operational risk with normal review. Evidenced by: Turns a postmortem's action items into shipped fixes rather than a filed document. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the incident-management standard other platform teams adopt. Defines the incident-command and postmortem practice several teams now run. Scope: incident leadership across a cross-team domain.</t>
+          <t>Depth: Independently leads severe incidents and drives durable remediation of risk. Evidenced by: Runs a major-incident review whose systemic fixes prevent the class of failure from recurring. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the incident-response operating model a sub-org relies on, from severity taxonomy to comms protocol and learning loop. Drives a measurable drop in MTTR or repeat incidents across the sub-org through the leaders who own each service. Scope: incident leadership across a platform sub-org.</t>
+          <t>Depth: Defines incident and risk practices others adopt and commands the worst crises calmly. Evidenced by: Defines the incident-command and postmortem practice several teams now run. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives the function's operational-excellence and reliability-leadership strategy. Sets the incident and reliability standard the function is accountable to. Scope: reliability leadership across the platform function.</t>
+          <t>Depth: Defines incident and risk practices others adopt and commands the worst crises calmly. Evidenced by: Drives a measurable drop in MTTR or repeat incidents across the sub-org through the leaders who own each service. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide incident-management and reliability-leadership model. Pioneers an operational-excellence practice other orgs reference. Scope: org-wide incident and reliability leadership.</t>
+          <t>Depth: Sets the org's operational-risk strategy and anticipates systemic failure modes. Evidenced by: Sets the incident and reliability standard the function is accountable to. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines what excellent operational risk management means and shapes external practice. Evidenced by: Pioneers an operational-excellence practice other orgs reference. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -1704,37 +1790,42 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Majors, Fong-Jones &amp; Miranda, Observability Engineering (2022)</t>
+          <t>Makes system behavior visible.</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Depth: Ensures the team's services are observable across metrics, logs, traces, and actionable alerts. Replaces a noisy or blind alert with a signal that maps to real user pain. Scope: observability for one platform team's services.</t>
+          <t>Majors, Fong-Jones &amp; Miranda, Observability Engineering: Achieving Production Excellence (O'Reilly, 2022) — you cannot operate or improve what you cannot see</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs the observability strategy for a critical platform area, including SLI instrumentation and high-cardinality debugging. Makes a previously opaque failure mode diagnosable in minutes. Scope: observability for a high-stakes platform team.</t>
+          <t>Depth: Instruments their services; builds dashboards; tunes alerts to limit noise. Evidenced by: Replaces a noisy or blind alert with a signal that maps to real user pain. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the observability standard other platform teams adopt. Defines the instrumentation and alerting baseline several teams now build to. Scope: observability across a cross-team domain.</t>
+          <t>Depth: Designs observability for complex systems (end-to-end traces, quality signals, cost attribution). Evidenced by: Makes a previously opaque failure mode diagnosable in minutes. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the observability platform and practice a sub-org runs on, controlling cost and cardinality. Makes health signals consistent and comparable across the sub-org's services. Scope: observability across a platform sub-org.</t>
+          <t>Depth: Expert in instrumentation trade-offs at scale, incl. privacy-safe logging. Evidenced by: Defines the instrumentation and alerting baseline several teams now build to. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives the function's observability strategy and its economics. Sets the observability standard the function commits to. Scope: observability across the platform function.</t>
+          <t>Depth: Expert in instrumentation trade-offs at scale, incl. privacy-safe logging. Evidenced by: Makes health signals consistent and comparable across the sub-org's services. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide observability model. Pioneers an approach to health signals other orgs adopt. Scope: org-wide observability.</t>
+          <t>Depth: Defines org observability strategy. Evidenced by: Sets the observability standard the function commits to. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Shapes company-wide operational visibility; advances practice. Evidenced by: Pioneers an approach to health signals other orgs adopt. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -1761,37 +1852,42 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Beyer, Jones, Petoff &amp; Murphy, Site Reliability Engineering (2016) - toil chapter</t>
+          <t>Default to eliminating toil by automating repetitive operational work.</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>Depth: Tracks the team's toil and automates the worst of it to protect engineering time. Converts a recurring manual operational task into an automated one. Scope: toil on one platform team.</t>
+          <t>Beyer, Jones, Petoff &amp; Murphy (eds.), Site Reliability Engineering: How Google Runs Production Systems (O'Reilly/Google, 2016) — unmanaged toil caps leverage; automating it is how platform scales sublinearly with load</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets a toil budget for a critical platform team and drives it down structurally. Cuts on-call and operational load enough to visibly change the team's toil ratio. Scope: toil for a high-stakes platform team.</t>
+          <t>Depth: Independently automates routine operational tasks and integrates them into standard workflows with normal review. Evidenced by: Converts a recurring manual operational task into an automated one. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the toil-measurement and automation standard other platform teams adopt. Defines the toil-budget practice several teams now manage their operational load with. Scope: toil reduction across a cross-team domain.</t>
+          <t>Depth: Designs automation for ambiguous, error-prone toil and resolves hard reliability and orchestration issues in pipelines. Evidenced by: Cuts on-call and operational load enough to visibly change the team's toil ratio. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the automation strategy a sub-org uses to keep operational cost sublinear as it scales. Drives a sub-org-wide reduction in toil through the platforms that eliminate it. Scope: automation leverage across a platform sub-org.</t>
+          <t>Depth: Defines automation patterns and toil-elimination practices others adopt, solving deep workflow and safety problems. Evidenced by: Defines the toil-budget practice several teams now manage their operational load with. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives the function's operational-leverage strategy, targeting where automation investment buys the most headroom. Sets the toil and automation targets the function commits to. Scope: operational leverage across the platform function.</t>
+          <t>Depth: Defines automation patterns and toil-elimination practices others adopt, solving deep workflow and safety problems. Evidenced by: Drives a sub-org-wide reduction in toil through the platforms that eliminate it. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide expectation that operations scale through automation, not headcount. Pioneers an operational-leverage model other orgs adopt. Scope: org-wide operational leverage.</t>
+          <t>Depth: Sets organization-wide automation strategy, anticipating where automation-first operations should head. Evidenced by: Sets the toil and automation targets the function commits to. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines what automation-first operations means for the discipline, externally credible in shaping the practice. Evidenced by: Pioneers an operational-leverage model other orgs adopt. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -1818,37 +1914,42 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Gregg, Systems Performance (2nd ed., 2020)</t>
+          <t>Keeps systems fast and economical.</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Depth: Watches the team's capacity, performance, and spend. Right-sizes a resource or fixes a performance regression to cut cost without hurting reliability. Scope: capacity and cost for one platform team's services.</t>
+          <t>Gregg, Systems Performance: Enterprise and the Cloud, 2nd ed. (Addison-Wesley, 2020) — capacity, performance, and cost are one coupled system, the FinOps lever of a platform</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>Depth: Owns capacity and cost planning for a critical platform area, forecasting demand and managing efficiency. Lands a material infrastructure-cost reduction while holding SLOs. Scope: capacity and FinOps for a high-stakes platform team.</t>
+          <t>Depth: Applies standard optimizations; stays within cost/latency budgets. Evidenced by: Right-sizes a resource or fixes a performance regression to cut cost without hurting reliability. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the capacity-planning and cost-efficiency standard other platform teams adopt. Defines the FinOps and performance practice several teams now manage spend with. Scope: capacity and cost across a cross-team domain.</t>
+          <t>Depth: Designs cost-aware architectures; defines and tracks unit economics for a domain. Evidenced by: Lands a material infrastructure-cost reduction while holding SLOs. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the capacity and FinOps operating model a sub-org runs on, from forecasting to unit economics and efficiency governance. Makes infrastructure unit cost a managed, trending metric across the sub-org. Scope: capacity and cost across a platform sub-org.</t>
+          <t>Depth: Expert in economics at scale (fleet optimization, build-vs-buy). Evidenced by: Defines the FinOps and performance practice several teams now manage spend with. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives the function's infrastructure-efficiency and cost strategy and its business framing. Sets the unit-economics and capacity commitments the function owns. Scope: capacity and FinOps across the platform function.</t>
+          <t>Depth: Expert in economics at scale (fleet optimization, build-vs-buy). Evidenced by: Makes infrastructure unit cost a managed, trending metric across the sub-org. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide infrastructure-efficiency posture and the company's cloud and capital strategy for platform. Pioneers a FinOps model the business plans spend around. Scope: org-wide capacity, performance, and cost.</t>
+          <t>Depth: Owns org-level spend strategy; cost decisions change margins. Evidenced by: Sets the unit-economics and capacity commitments the function owns. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Shapes the company economics of the products. Evidenced by: Pioneers a FinOps model the business plans spend around. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -1875,37 +1976,42 @@
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Conway (1968); Nygard, Documenting Architecture Decisions (2011)</t>
+          <t>Evaluates and justifies design options against competing quality attributes and constraints.</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Depth: Stewards the team's platform architecture and keeps decisions recorded as ADRs. Catches an architectural drift or coupling problem in review before it ships. Scope: architecture for one platform team's surface.</t>
+          <t>Conway, How Do Committees Invent?, Datamation 14(4), 28-31 (1968) — platform architecture and org design are coupled, and decisions must be recorded to hold coherence</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>Depth: Owns architectural direction for a critical platform area, weighing evolvability and Conway-aligned boundaries. Redesigns a component boundary so team and system seams line up. Scope: architecture for a high-stakes platform team.</t>
+          <t>Depth: Evaluates standard trade-offs independently for routine architectural choices. Evidenced by: Catches an architectural drift or coupling problem in review before it ships. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the architecture and ADR standard other platform teams adopt. Defines the reference architecture and decision-record practice several teams now build within. Scope: architecture stewardship across a cross-team domain.</t>
+          <t>Depth: Structures and defends trade-off decisions for ambiguous, high-stakes designs autonomously. Evidenced by: Redesigns a component boundary so team and system seams line up. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the architecture-governance model a sub-org runs on, from review forums to principles and Conway-aware team-and-system design. Shapes a sub-org's team topology to fit the platform architecture it needs. Scope: architecture across a platform sub-org.</t>
+          <t>Depth: Defines trade-off analysis methods and decision frameworks others adopt. Evidenced by: Defines the reference architecture and decision-record practice several teams now build within. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives the function's architectural direction and its long-horizon coherence. Sets the architecture principles the function builds against. Scope: architecture across the platform function.</t>
+          <t>Depth: Defines trade-off analysis methods and decision frameworks others adopt. Evidenced by: Shapes a sub-org's team topology to fit the platform architecture it needs. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide platform-architecture vision and the socio-technical structure to realize it. Pioneers an architecture other orgs study. Scope: org-wide platform architecture.</t>
+          <t>Depth: Sets how the organization makes architectural trade-offs, anticipating future tensions. Evidenced by: Sets the architecture principles the function builds against. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Advances trade-off-analysis practice recognized across the industry. Evidenced by: Pioneers an architecture other orgs study. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -1932,37 +2038,42 @@
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>Humble &amp; Farley, Continuous Delivery (2010)</t>
+          <t>Keeps code healthy, modular and maintainable.</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Depth: Holds the team to engineering standards across CI, testing, code review, and deployment safety. Raises a slipping quality practice such as test coverage or review rigor on the team. Scope: standards on one platform team.</t>
+          <t>Humble &amp; Farley, Continuous Delivery: Reliable Software Releases through Build Test and Deployment Automation (Addison-Wesley, 2010) — quality is built in through automation and standards, not inspected in afterward</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the quality bar for a critical platform team, including continuous delivery, progressive delivery, and change safety. Installs a delivery-safety practice that measurably cuts change-failure rate. Scope: standards for a high-stakes platform team.</t>
+          <t>Depth: Writes clean, documented, modular code; gives useful review feedback. Evidenced by: Raises a slipping quality practice such as test coverage or review rigor on the team. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the engineering-standards baseline other platform teams adopt. Defines the CI/CD and quality standard several teams now build to. Scope: standards across a cross-team domain.</t>
+          <t>Depth: Designs for maintainability; leads refactors of problem areas; review feedback teaches. Evidenced by: Installs a delivery-safety practice that measurably cuts change-failure rate. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the engineering-excellence model a sub-org runs on, from golden paths for quality to paved CI/CD and standards governance. Makes high-quality delivery the default path across the sub-org. Scope: standards across a platform sub-org.</t>
+          <t>Depth: Expert in code health at scale (shared libraries, deprecations, large migrations). Evidenced by: Defines the CI/CD and quality standard several teams now build to. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives the function's engineering-quality strategy and its link to delivery performance. Sets the quality standard the function commits to. Scope: standards across the platform function.</t>
+          <t>Depth: Expert in code health at scale (shared libraries, deprecations, large migrations). Evidenced by: Makes high-quality delivery the default path across the sub-org. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K22" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide engineering-quality bar. Pioneers a standards model other functions adopt. Scope: org-wide engineering standards.</t>
+          <t>Depth: Shapes org-wide engineering standards for long-lived codebases. Evidenced by: Sets the quality standard the function commits to. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines what good engineering looks like company-wide; externally recognized. Evidenced by: Pioneers a standards model other functions adopt. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -1989,37 +2100,42 @@
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Cunningham, The WyCash Portfolio Management System (1992)</t>
+          <t>Surfaces, prices, and manages technical debt and technical risk as an economic portfolio — funding paydown structurally and setting the speed-versus-soundness posture explicitly.</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>Depth: Tracks the team's tech debt and budgets time to pay it down deliberately. Makes a debt trade-off explicit in planning rather than letting it accrue silently. Scope: debt on one platform team.</t>
+          <t>Cunningham, The WyCash Portfolio Management System, OOPSLA 1992 Experience Report — debt is a deliberate liability with interest, paid down on purpose, not neglected mess</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>Depth: Manages debt and modernization for a critical platform area, sequencing paydown against risk. Funds and lands a modernization that removes a systemic drag on the team. Scope: debt for a high-stakes platform team.</t>
+          <t>Depth: Keeps a visible debt register with the cost of carry noted and defends a steady paydown allocation in planning rather than begging quarter by quarter. Evidenced by: Makes a debt trade-off explicit in planning rather than letting it accrue silently. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the debt-management standard other platform teams adopt. Defines the debt-accounting and modernization practice several teams now prioritize with. Scope: debt strategy across a cross-team domain.</t>
+          <t>Depth: Distinguishes debt worth carrying from debt that will detonate, sequences remediation by risk, and prices debt in incident and velocity terms stakeholders accept. Evidenced by: Funds and lands a modernization that removes a systemic drag on the team. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the modernization roadmap a sub-org runs on, balancing debt paydown against new capability. Wins sustained investment for a sub-org-wide modernization others deprioritized. Scope: modernization across a platform sub-org.</t>
+          <t>Depth: Makes debt legible across multiple teams — shared taxonomy, reporting rhythm — and gets cross-team risk (the shared library nobody owns, the half-finished migration) owned and funded. Evidenced by: Defines the debt-accounting and modernization practice several teams now prioritize with. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives the function's technical-health and modernization strategy. Sets the debt and modernization commitments the function makes. Scope: technical health across the platform function.</t>
+          <t>Depth: Makes debt legible across multiple teams — shared taxonomy, reporting rhythm — and gets cross-team risk (the shared library nobody owns, the half-finished migration) owned and funded. Evidenced by: Wins sustained investment for a sub-org-wide modernization others deprioritized. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide posture on technical debt and legacy modernization. Pioneers a debt-management model the business funds against. Scope: org-wide modernization.</t>
+          <t>Depth: Carries technical risk onto the executive risk register — top exposures known, sized, owned, trending — and lands multi-quarter remediation programs against feature pressure. Evidenced by: Sets the debt and modernization commitments the function makes. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Sets an organization's speed-versus-soundness posture explicitly — where debt is accepted for velocity and where it never is — and holds it under growth pressure. Evidenced by: Pioneers a debt-management model the business funds against. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -2046,37 +2162,42 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Larson, An Elegant Puzzle (2019); Wardley Maps (2016)</t>
+          <t>Shapes technical direction beyond own work.</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>Depth: Connects the team's technical choices to a coherent direction. Frames a build decision as a bet with a stated rationale, not an ad-hoc pick. Scope: technical direction for one platform team.</t>
+          <t>Larson, An Elegant Puzzle: Systems of Engineering Management (Stripe Press, 2019) — technical strategy is placing a few high-leverage bets and mapping where value sits</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets multi-quarter technical strategy for a critical platform area, sequencing investment by leverage. Makes a hard technical-investment call such as rebuild versus extend and defends it with evidence. Scope: technical strategy for a high-stakes platform team.</t>
+          <t>Depth: Influences component-level decisions through credibility. Evidenced by: Frames a build decision as a bet with a stated rationale, not an ad-hoc pick. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets a cross-team technical strategy other teams align to. Publishes a domain technical strategy or Wardley map that redirects where several teams invest. Scope: technical strategy across a cross-team domain.</t>
+          <t>Depth: Sets technical direction for a domain; others align to their calls. Evidenced by: Makes a hard technical-investment call such as rebuild versus extend and defends it with evidence. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the technical-investment thesis a sub-org executes, deciding where to concentrate platform bets over years. Frames the small set of bets the sub-org organizes its roadmap around. Scope: technical strategy across a platform sub-org.</t>
+          <t>Depth: Shapes how multiple teams approach problems; trusted tiebreaker. Evidenced by: Publishes a domain technical strategy or Wardley map that redirects where several teams invest. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives the function's technical strategy and its alignment to business strategy. Sets the technology bets the function commits capital and headcount to. Scope: technical strategy across the platform function.</t>
+          <t>Depth: Shapes how multiple teams approach problems; trusted tiebreaker. Evidenced by: Frames the small set of bets the sub-org organizes its roadmap around. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K24" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide platform-technology direction and the long-horizon infrastructure bets. Pioneers a technical strategy the company's product strategy depends on. Scope: org-wide technical strategy.</t>
+          <t>Depth: Influences org-wide technical strategy. Evidenced by: Sets the technology bets the function commits capital and headcount to. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Influences company strategic direction through insight. Evidenced by: Pioneers a technical strategy the company's product strategy depends on. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -2103,37 +2224,42 @@
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Korn Ferry Leadership Architect (2014) - Financial Acumen</t>
+          <t>Managing budgets, costs, and external vendor or contractor relationships.</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>Depth: Makes build/buy/adopt calls for the team's tooling with a stated cost and benefit. Avoids building something a supported off-the-shelf option already solves. Scope: build/buy for one platform team.</t>
+          <t>Korn Ferry, Korn Ferry Leadership Architect Global Competency Framework (2014) — build-vs-buy and vendor choices are capital-allocation decisions needing financial judgment</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs build/buy/adopt and vendor evaluations for a critical platform area, including total cost of ownership and lock-in risk. Negotiates or selects a platform vendor on a defensible total-cost basis. Scope: build/buy for a high-stakes platform team.</t>
+          <t>Depth: Manages a team budget and standard vendor relationships with normal review. Evidenced by: Avoids building something a supported off-the-shelf option already solves. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the build/buy/adopt decision standard other platform teams use. Defines the evaluation and vendor-selection framework several teams now decide with. Scope: sourcing strategy across a cross-team domain.</t>
+          <t>Depth: Independently controls budgets under pressure and negotiates difficult vendor terms. Evidenced by: Negotiates or selects a platform vendor on a defensible total-cost basis. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the vendor and sourcing strategy a sub-org runs on, managing the platform supplier portfolio and consolidation. Drives a sub-org-wide build-versus-buy decision with material budget impact. Scope: sourcing across a platform sub-org.</t>
+          <t>Depth: Defines budget and vendor practices others adopt and rescues failing vendor relationships. Evidenced by: Defines the evaluation and vendor-selection framework several teams now decide with. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives the function's build/buy and vendor strategy and its capital implications. Sets the sourcing principles and major vendor relationships the function commits to. Scope: sourcing across the platform function.</t>
+          <t>Depth: Defines budget and vendor practices others adopt and rescues failing vendor relationships. Evidenced by: Drives a sub-org-wide build-versus-buy decision with material budget impact. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide platform build-versus-buy posture and negotiates strategic supplier relationships. Pioneers a sourcing strategy the business plans capital around. Scope: org-wide sourcing and vendor strategy.</t>
+          <t>Depth: Sets org-wide budget and vendor strategy and anticipates cost and supplier risks. Evidenced by: Sets the sourcing principles and major vendor relationships the function commits to. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines exemplary budget and vendor management for the field and influences practice. Evidenced by: Pioneers a sourcing strategy the business plans capital around. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -2160,37 +2286,42 @@
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>OWASP, Application Security Verification Standard (v4, 2019)</t>
+          <t>Encodes preventive controls as versioned, tested, automatically enforced policy - admission checks, pipeline gates, configuration rules - with actionable violation messages and governed exception paths, so the safe way is the default way.</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>Depth: Holds the team to security and compliance baselines. Bakes a security control into the platform so users get it by default rather than bolting it on. Scope: security posture for one platform team's surface.</t>
+          <t>OWASP Foundation, OWASP Application Security Verification Standard (accessed 2026-07) — platforms are the leverage point where security is built in for everyone or absent for everyone</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>Depth: Owns the security and compliance posture for a critical platform area, managing risk and remediation. Closes a systemic vulnerability class through a platform control rather than one-off fixes. Scope: security for a high-stakes platform team.</t>
+          <t>Depth: Writes and tests policy rules for a component - admission checks, pipeline gates - with low false-positive rates and violation messages that tell the user how to comply. Evidenced by: Bakes a security control into the platform so users get it by default rather than bolting it on. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the security and compliance standard other platform teams adopt. Defines the paved-road security controls several teams now inherit by default. Scope: security posture across a cross-team domain.</t>
+          <t>Depth: Designs the guardrail architecture for a capability - what is blocked, warned, or audited, with documented threat reasoning - tuned so the safe path is the fast path, and runs an audited exception workflow without becoming the bottleneck. Evidenced by: Closes a systemic vulnerability class through a platform control rather than one-off fixes. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the security and compliance operating model a sub-org runs on, from controls-as-code to audit readiness and risk governance. Makes secure-by-default the path of least resistance across the sub-org. Scope: security across a platform sub-org.</t>
+          <t>Depth: Harmonizes policy across teams into a coherent, versioned policy library with a governed exception process, and adjudicates escalated safety-versus-velocity disputes. Evidenced by: Defines the paved-road security controls several teams now inherit by default. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives the function's security and risk strategy and its regulatory posture. Sets the risk commitments and compliance guarantees the function owns. Scope: security across the platform function.</t>
+          <t>Depth: Harmonizes policy across teams into a coherent, versioned policy library with a governed exception process, and adjudicates escalated safety-versus-velocity disputes. Evidenced by: Makes secure-by-default the path of least resistance across the sub-org. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide platform-security and risk posture. Pioneers a secure-platform model auditors and peers reference. Scope: org-wide security and risk.</t>
+          <t>Depth: Owns an organization's preventive-control strategy with security partners - the control catalog, its coverage, and the evidence it works - moving enforcement from review-time to platform-time. Evidenced by: Sets the risk commitments and compliance guarantees the function owns. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Sets an organization-defining balance of enablement and control, accountable for guardrails that hold under audit and attack without throttling delivery. Evidenced by: Pioneers a secure-platform model auditors and peers reference. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -2217,37 +2348,42 @@
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>McConnell, Software Estimation (2006)</t>
+          <t>Forecasts and plans work credibly.</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs the team's planning with realistic, range-based estimates. Surfaces a schedule risk early instead of discovering the slip at the deadline. Scope: planning for one platform team.</t>
+          <t>McConnell, Software Estimation: Demystifying the Black Art (Microsoft Press, 2006) — estimation is a probabilistic forecast to calibrate, not a promise, and platform work is especially uncertain</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>Depth: Plans complex, cross-dependent platform work with calibrated estimates and buffers. Replans a high-stakes platform delivery mid-flight without losing the commitment. Scope: planning for a critical platform team.</t>
+          <t>Depth: Estimates scoped work realistically; plans own 1-3 week projects. Evidenced by: Surfaces a schedule risk early instead of discovering the slip at the deadline. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the planning and estimation standard other platform teams adopt. Defines the forecasting practice several teams now plan with. Scope: planning across a cross-team domain.</t>
+          <t>Depth: Plans quarter-scale, multi-workstream efforts including dependencies. Evidenced by: Replans a high-stakes platform delivery mid-flight without losing the commitment. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the planning operating model a sub-org runs on, from commitment framing to capacity-based forecasting and uncertainty comms. Makes sub-org delivery forecasts credible to stakeholders. Scope: planning across a platform sub-org.</t>
+          <t>Depth: Expert at planning large programs; anticipates risk early. Evidenced by: Defines the forecasting practice several teams now plan with. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives the function's planning cadence and its integration with company planning. Sets the planning discipline the function commits to. Scope: planning across the platform function.</t>
+          <t>Depth: Expert at planning large programs; anticipates risk early. Evidenced by: Makes sub-org delivery forecasts credible to stakeholders. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K27" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide planning model for platform investment. Pioneers a forecasting practice other functions adopt. Scope: org-wide platform planning.</t>
+          <t>Depth: Plans org-level programs across quarters/years. Evidenced by: Sets the planning discipline the function commits to. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Shapes how the company plans major technical change. Evidenced by: Pioneers a forecasting practice other functions adopt. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -2274,37 +2410,42 @@
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>Reinertsen, The Principles of Product Development Flow (2009)</t>
+          <t>Weighs cost, value, risk and timing.</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>Depth: Prioritizes the team's backlog against value and urgency. Says no to a low-value request with a clear rationale rather than absorbing everything. Scope: prioritization for one platform team.</t>
+          <t>Reinertsen, The Principles of Product Development Flow: Second Generation Lean Product Development (Celeritas, 2009) — prioritizing by cost of delay and managing queues, not utilization, maximizes economic flow</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>Depth: Makes hard prioritization calls for a critical platform area using cost-of-delay thinking. Defends a contested platform trade-off between competing stakeholder demands. Scope: prioritization for a high-stakes platform team.</t>
+          <t>Depth: Makes sound priority calls within scope; time-boxes uncertain work. Evidenced by: Says no to a low-value request with a clear rationale rather than absorbing everything. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the prioritization framework other platform teams adopt. Installs a cost-of-delay or WSJF practice several teams now sequence with. Scope: prioritization across a cross-team domain.</t>
+          <t>Depth: Balances cost/value/risk across a domain; resists hype; decisions hold up over months. Evidenced by: Defends a contested platform trade-off between competing stakeholder demands. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the portfolio-prioritization model a sub-org allocates by, balancing platform bets against keep-the-lights-on. Arbitrates a sub-org-wide trade-off that reallocates investment. Scope: prioritization across a platform sub-org.</t>
+          <t>Depth: Expert at portfolio-level trade-offs; surfaces hidden assumptions; trusted tiebreaker. Evidenced by: Installs a cost-of-delay or WSJF practice several teams now sequence with. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives how the function prioritizes across competing business demands. Sets the prioritization principles the function commits capacity against. Scope: prioritization across the platform function.</t>
+          <t>Depth: Expert at portfolio-level trade-offs; surfaces hidden assumptions; trusted tiebreaker. Evidenced by: Arbitrates a sub-org-wide trade-off that reallocates investment. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K28" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide framework for prioritizing platform investment. Pioneers a portfolio-prioritization model other functions adopt. Scope: org-wide prioritization.</t>
+          <t>Depth: Sets decision frameworks for the org. Evidenced by: Sets the prioritization principles the function commits capacity against. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Influences company strategic direction through judgment. Evidenced by: Pioneers a portfolio-prioritization model other functions adopt. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -2331,37 +2472,42 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Brooks, The Mythical Man-Month (1975)</t>
+          <t>Forecasting staffing needs and allocating people across initiatives and priorities.</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>Depth: Allocates the team's capacity across roadmap, on-call, and interrupts. Protects focus time rather than fragmenting the team across too many fronts. Scope: capacity for one platform team.</t>
+          <t>Brooks, The Mythical Man-Month: Essays on Software Engineering, Anniversary ed. (Addison-Wesley, 1995; orig. 1975) — people and time do not trade linearly, so allocation is a judgment lever</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>Depth: Balances capacity for a critical platform team across delivery, reliability, and toil. Rebalances staffing to unblock a priority without wrecking sustainability. Scope: capacity for a high-stakes platform team.</t>
+          <t>Depth: Builds a credible headcount plan for one team with normal review. Evidenced by: Protects focus time rather than fragmenting the team across too many fronts. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the capacity-allocation standard other platform leads use. Defines the staffing and load-balancing model several teams now allocate with. Scope: allocation across a cross-team domain.</t>
+          <t>Depth: Independently plans resourcing under uncertainty and defends staffing trade-offs. Evidenced by: Rebalances staffing to unblock a priority without wrecking sustainability. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the resource-allocation model a sub-org runs on, mapping headcount to bets with realistic ramp and no linear-scaling assumptions. Reallocates capacity across a sub-org to match investment shifts. Scope: allocation across a platform sub-org.</t>
+          <t>Depth: Defines resource-planning practices others adopt and resolves cross-team allocation conflicts. Evidenced by: Defines the staffing and load-balancing model several teams now allocate with. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives how the function allocates headcount against strategy. Sets the resourcing principles the function plans against. Scope: allocation across the platform function.</t>
+          <t>Depth: Defines resource-planning practices others adopt and resolves cross-team allocation conflicts. Evidenced by: Reallocates capacity across a sub-org to match investment shifts. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K29" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide model for allocating platform capacity. Pioneers a resourcing approach other functions adopt. Scope: org-wide capacity allocation.</t>
+          <t>Depth: Sets org-wide resourcing strategy and anticipates future capacity demand. Evidenced by: Sets the resourcing principles the function plans against. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines headcount-planning best practice for the discipline and is recognized for it. Evidenced by: Pioneers a resourcing approach other functions adopt. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -2388,37 +2534,42 @@
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>Forsgren, Humble &amp; Kim, Accelerate (2018)</t>
+          <t>Driving cross-team execution, dependencies, and predictable delivery of programs.</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs the team to a predictable delivery cadence with small batches. Removes a recurring flow blocker such as a handoff, review lag, or big-batch release that stalls delivery. Scope: delivery flow for one platform team.</t>
+          <t>Forsgren, Humble &amp; Kim, Accelerate: The Science of Lean Software and DevOps (IT Revolution Press, 2018) — predictable, high-frequency delivery is an engineered property that predicts org performance</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>Depth: Engineers predictable delivery for a critical platform team under real operational load. Stabilizes a team's delivery so its commitments become trustworthy. Scope: flow for a high-stakes platform team.</t>
+          <t>Depth: Drives delivery of a standard program with normal review. Evidenced by: Removes a recurring flow blocker such as a handoff, review lag, or big-batch release that stalls delivery. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the delivery-flow standard other platform teams adopt. Defines the flow and batch-size practice several teams now deliver with. Scope: delivery flow across a cross-team domain.</t>
+          <t>Depth: Independently runs complex multi-team programs and recovers slipping delivery. Evidenced by: Stabilizes a team's delivery so its commitments become trustworthy. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the delivery operating model a sub-org runs on, from flow metrics to dependency management and cadence. Makes a sub-org's delivery predictable through the leaders who run each team. Scope: flow across a platform sub-org.</t>
+          <t>Depth: Defines delivery practices others adopt and rescues the most troubled programs. Evidenced by: Defines the flow and batch-size practice several teams now deliver with. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives the function's delivery performance and its link to business outcomes. Sets the flow and predictability standard the function commits to. Scope: delivery across the platform function.</t>
+          <t>Depth: Defines delivery practices others adopt and rescues the most troubled programs. Evidenced by: Makes a sub-org's delivery predictable through the leaders who run each team. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K30" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide expectation for delivery performance. Pioneers a flow model other functions adopt. Scope: org-wide delivery flow.</t>
+          <t>Depth: Sets the org's delivery strategy and anticipates systemic delivery risks. Evidenced by: Sets the flow and predictability standard the function commits to. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines what excellent program delivery means and shapes external practice. Evidenced by: Pioneers a flow model other functions adopt. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -2445,37 +2596,42 @@
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>Forsgren, Humble &amp; Kim, Accelerate (2018) - DORA four keys; SPACE (2021)</t>
+          <t>Using delivery and health metrics to diagnose and improve team effectiveness.</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>Depth: Tracks the team's DORA and SPACE signals and uses them to improve, not to rank people. Acts on a delivery-metric trend to fix an actual bottleneck. Scope: metrics for one platform team.</t>
+          <t>Forsgren, Humble &amp; Kim, Accelerate: The Science of Lean Software and DevOps (IT Revolution Press, 2018) — DORA and SPACE give a validated, hard-to-game way to measure delivery, used to improve not to rank</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs a metrics practice for a critical platform team that resists gaming and connects to outcomes. Diagnoses a delivery-health problem from the four keys and fixes its root cause. Scope: metrics for a high-stakes platform team.</t>
+          <t>Depth: Interprets productivity metrics for one team with normal review. Evidenced by: Acts on a delivery-metric trend to fix an actual bottleneck. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the delivery-metrics standard other platform teams adopt. Defines the DORA and SPACE measurement several teams now steer by. Scope: metrics across a cross-team domain.</t>
+          <t>Depth: Independently designs metric systems and distinguishes real signal from vanity numbers. Evidenced by: Diagnoses a delivery-health problem from the four keys and fixes its root cause. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the delivery-health measurement system a sub-org runs on, making metrics comparable and honest. Makes data-driven delivery improvement the norm across the sub-org. Scope: metrics across a platform sub-org.</t>
+          <t>Depth: Defines the productivity-measurement model others adopt and debunks misleading metrics. Evidenced by: Defines the DORA and SPACE measurement several teams now steer by. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives how the function measures and reports delivery and developer productivity to the business. Sets the metrics the function commits to and defends against misuse. Scope: metrics across the platform function.</t>
+          <t>Depth: Defines the productivity-measurement model others adopt and debunks misleading metrics. Evidenced by: Makes data-driven delivery improvement the norm across the sub-org. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K31" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide definition of engineering delivery health. Pioneers a measurement model other functions adopt. Scope: org-wide delivery metrics.</t>
+          <t>Depth: Sets the org's engineering-metrics strategy and anticipates which signals will matter. Evidenced by: Sets the metrics the function commits to and defends against misuse. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines rigorous engineering productivity measurement and influences the field externally. Evidenced by: Pioneers a measurement model other functions adopt. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -2502,37 +2658,42 @@
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>Deming, Out of the Crisis (1986)</t>
+          <t>Designing rituals, workflows, and cadences that keep teams effective and aligned.</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs retros that produce real changes. Removes a wasteful step from the team's process instead of adding ceremony. Scope: process for one platform team.</t>
+          <t>Deming, Out of the Crisis (MIT Center for Advanced Engineering Study, 1986) — throughput comes from improving the system, not exhorting people</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives systemic process improvement on a critical platform team, attacking causes not symptoms. Lands a process change that measurably improves throughput or quality. Scope: process for a high-stakes platform team.</t>
+          <t>Depth: Runs and tunes a team's operating cadence with normal review. Evidenced by: Removes a wasteful step from the team's process instead of adding ceremony. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the continuous-improvement practice other platform teams adopt. Installs an improvement discipline several teams now run. Scope: improvement across a cross-team domain.</t>
+          <t>Depth: Independently designs processes that fit the work and removes friction others miss. Evidenced by: Lands a process change that measurably improves throughput or quality. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the operating rhythm and improvement system a sub-org runs on. Makes systematic improvement, not firefighting, the sub-org's default mode. Scope: process across a platform sub-org.</t>
+          <t>Depth: Defines operating-cadence patterns others adopt and fixes broken processes across teams. Evidenced by: Installs an improvement discipline several teams now run. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives the function's operating model and its improvement discipline. Sets the process standards the function runs on. Scope: process across the platform function.</t>
+          <t>Depth: Defines operating-cadence patterns others adopt and fixes broken processes across teams. Evidenced by: Makes systematic improvement, not firefighting, the sub-org's default mode. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K32" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide operating model for platform. Pioneers a continuous-improvement practice other functions adopt. Scope: org-wide process.</t>
+          <t>Depth: Sets the org's operating model and anticipates where cadence must evolve. Evidenced by: Sets the process standards the function runs on. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines effective engineering operating cadence for the discipline and is recognized for it. Evidenced by: Pioneers a continuous-improvement practice other functions adopt. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -2559,37 +2720,42 @@
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>NIST Cybersecurity Framework (2014); PMI PMBOK (2021)</t>
+          <t>Identify, assess, treat, and monitor risks across the organization within a risk appetite.</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>Depth: Tracks the team's dependencies and risks. Flags and mitigates a cross-team dependency before it blocks delivery. Scope: dependencies for one platform team.</t>
+          <t>NIST, The NIST Cybersecurity Framework (CSF) 2.0, NIST CSWP 29 (2024) — platforms sit on everyone else's critical path, so cross-team dependency and risk work is core</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>Depth: Manages complex cross-team dependencies and risk for a critical platform. Unblocks a delivery stalled on another team's dependency through negotiation, not escalation alone. Scope: dependencies for a high-stakes platform team.</t>
+          <t>Depth: Conducts standard risk assessments and updates registers independently with normal review. Evidenced by: Flags and mitigates a cross-team dependency before it blocks delivery. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the dependency and risk-management standard other platform teams adopt. Defines the cross-team dependency and risk practice several teams now coordinate with. Scope: dependency management across a cross-team domain.</t>
+          <t>Depth: Assesses complex, interconnected enterprise risks and sets local methodology autonomously. Evidenced by: Unblocks a delivery stalled on another team's dependency through negotiation, not escalation alone. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the risk and dependency-governance model a sub-org runs on, from risk registers to mitigation ownership and cross-team coordination. De-risks a sub-org-wide initiative with many moving dependencies. Scope: risk across a platform sub-org.</t>
+          <t>Depth: Designs the enterprise risk framework and appetite model others adopt; solves the hardest risk problems. Evidenced by: Defines the cross-team dependency and risk practice several teams now coordinate with. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives the function's approach to systemic and platform-wide risk. Sets the risk-management standard the function is accountable to. Scope: risk across the platform function.</t>
+          <t>Depth: Designs the enterprise risk framework and appetite model others adopt; solves the hardest risk problems. Evidenced by: De-risks a sub-org-wide initiative with many moving dependencies. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K33" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide model for managing platform and infrastructure risk. Pioneers a risk practice other functions adopt. Scope: org-wide risk and dependencies.</t>
+          <t>Depth: Sets enterprise risk strategy and appetite at board level; anticipates emerging systemic risks. Evidenced by: Sets the risk-management standard the function is accountable to. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines enterprise-risk practice recognized industry-wide; externally cited authority. Evidenced by: Pioneers a risk practice other functions adopt. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -2616,37 +2782,42 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>Rumelt, Good Strategy Bad Strategy (2011)</t>
+          <t>Define enterprise direction, scope, and competitive positioning to create durable advantage.</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>Depth: Frames the team's direction as a real strategy of diagnosis, guiding policy, and action. Names the core problem the team's strategy actually addresses rather than listing goals. Scope: strategy for one platform team.</t>
+          <t>Rumelt, Good Strategy Bad Strategy: The Difference and Why It Matters (Crown Business, 2011) — real strategy is a diagnosis plus a coherent guiding policy and actions, not a list of goals</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>Depth: Formulates strategy for a critical platform area with a sharp diagnosis and honest trade-offs. Produces a platform strategy that says no to things, not just yes. Scope: strategy for a high-stakes platform team.</t>
+          <t>Depth: Develops components of strategy and standard analyses independently with normal review. Evidenced by: Names the core problem the team's strategy actually addresses rather than listing goals. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets a cross-team platform strategy others align to. Publishes a domain strategy several teams reorient their plans around. Scope: strategy across a cross-team domain.</t>
+          <t>Depth: Frames ambiguous strategic problems and shapes coherent strategy autonomously; the go-to strategist. Evidenced by: Produces a platform strategy that says no to things, not just yes. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives strategy for a platform sub-org, integrating multiple domains into one coherent guiding policy. Builds a sub-org strategy that survives exec scrutiny and reallocates real investment. Scope: strategy across a platform sub-org.</t>
+          <t>Depth: Defines strategy-formulation approaches others adopt; resolves the hardest strategic trade-offs. Evidenced by: Publishes a domain strategy several teams reorient their plans around. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives the function's strategy and its coupling to company strategy. Sets the strategic bets the function commits to and defends them at the top table. Scope: strategy across the platform function.</t>
+          <t>Depth: Sets the enterprise strategic direction; anticipates major shifts reshaping the competitive landscape. Evidenced by: Builds a sub-org strategy that survives exec scrutiny and reallocates real investment. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K34" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide platform strategy. Pioneers a strategic thesis the company's direction depends on. Scope: org-wide platform strategy.</t>
+          <t>Depth: Sets the enterprise strategic direction; anticipates major shifts reshaping the competitive landscape. Evidenced by: Sets the strategic bets the function commits to and defends them at the top table. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L34" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines corporate-strategy practice recognized industry-wide; externally cited thought leader. Evidenced by: Pioneers a strategic thesis the company's direction depends on. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -2673,37 +2844,42 @@
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>Kotter, Leading Change (1996)</t>
+          <t>Leading teams through reorganization, process change, and shifting priorities.</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>Depth: Leads change on the team by building buy-in, not decree. Gets a team through a tooling or process change without losing people or momentum. Scope: change on one platform team.</t>
+          <t>Kotter, Leading Change (Harvard Business School Press, 1996) — durable change needs urgency, coalition, and follow-through, not a mandate</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives a significant change on a critical platform team against resistance. Builds the coalition that makes a hard platform migration or reorg stick. Scope: change for a high-stakes platform team.</t>
+          <t>Depth: Leads a contained team change with normal review. Evidenced by: Gets a team through a tooling or process change without losing people or momentum. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the change-leadership approach other platform leads adopt. Drives a cross-team transformation through the leaders who own each team. Scope: change across a cross-team domain.</t>
+          <t>Depth: Independently drives significant change through resistance to durable adoption. Evidenced by: Builds the coalition that makes a hard platform migration or reorg stick. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Depth: Leads sub-org-wide transformation, sequencing urgency, coalition, and consolidation. Lands a sub-org change that outlives the initial push. Scope: change across a platform sub-org.</t>
+          <t>Depth: Defines change approaches others adopt and rescues stalled transformations. Evidenced by: Drives a cross-team transformation through the leaders who own each team. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives change across the function and into its partner orgs. Sets the change the function leads and sustains. Scope: change across the platform function.</t>
+          <t>Depth: Defines change approaches others adopt and rescues stalled transformations. Evidenced by: Lands a sub-org change that outlives the initial push. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K35" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets and leads org-wide platform transformation. Pioneers a change other functions model theirs on. Scope: org-wide transformation.</t>
+          <t>Depth: Sets the org's transformation strategy and anticipates where change is needed next. Evidenced by: Sets the change the function leads and sustains. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines effective engineering transformation for the discipline and shapes external practice. Evidenced by: Pioneers a change other functions model theirs on. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -2730,37 +2906,42 @@
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>Skelton &amp; Pais, Team Topologies (2019); Conway (1968)</t>
+          <t>Shaping team topologies, roles, and reporting lines to fit the work and scale.</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>Depth: Shapes the team's roles, boundaries, and interaction modes deliberately. Clarifies a fuzzy team boundary that was causing thrash. Scope: team design for one platform team.</t>
+          <t>Skelton &amp; Pais, Team Topologies (IT Revolution, 2019) — team boundaries shape the software, and platform teams exist to cut others' cognitive load</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs the structure of a critical platform team and its interaction modes, whether X-as-a-service or collaboration. Restructures a team so its boundary matches the platform it owns. Scope: team design for a high-stakes platform team.</t>
+          <t>Depth: Designs a sound structure for one team with normal review. Evidenced by: Clarifies a fuzzy team boundary that was causing thrash. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the team-topology approach other platform leads adopt. Redesigns team boundaries across the domain to cut cross-team cognitive load. Scope: org design across a cross-team domain.</t>
+          <t>Depth: Independently restructures teams to fit changing work and resolves boundary conflicts. Evidenced by: Restructures a team so its boundary matches the platform it owns. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs the org structure of a platform sub-org using stream-aligned, platform, and enabling patterns. Proposes and drives a sub-org reshape that improves flow. Scope: org design across a platform sub-org.</t>
+          <t>Depth: Defines org-design approaches others adopt and reshapes the most tangled structures. Evidenced by: Redesigns team boundaries across the domain to cut cross-team cognitive load. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives the function's org design and its Conway-aligned interfaces to product orgs. Sets the operating structure the function runs on. Scope: org design across the platform function.</t>
+          <t>Depth: Defines org-design approaches others adopt and reshapes the most tangled structures. Evidenced by: Proposes and drives a sub-org reshape that improves flow. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K36" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide socio-technical structure for platform. Pioneers an operating model other functions adopt. Scope: org-wide org design.</t>
+          <t>Depth: Sets org-structuring strategy across the org and anticipates scaling inflection points. Evidenced by: Sets the operating structure the function runs on. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L36" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines effective engineering-org design for the discipline and is cited externally on it. Evidenced by: Pioneers an operating model other functions adopt. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -2787,37 +2968,42 @@
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>Duarte, HBR Guide to Persuasive Presentations (2012)</t>
+          <t>Communicates upward and to executive audiences — answer-first briefings, decision-ready framing, and composure under hostile questioning.</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>Depth: Communicates the team's work clearly to stakeholders, tuned to the audience. Translates a technical platform issue into terms a non-engineer decision-maker acts on. Scope: communication for one platform team.</t>
+          <t>Duarte, HBR Guide to Persuasive Presentations (Harvard Business Review Press, 2012) — leaders move resources through clear, audience-tuned narrative, not data dumps</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>Depth: Represents a critical platform area to senior stakeholders with a clear narrative under scrutiny. Gets a skeptical stakeholder to a decision through a well-framed case. Scope: communication for a high-stakes platform team.</t>
+          <t>Depth: Reports upward answer-first with a specific ask; escalates early with options attached, so no surprise reaches leadership from someone else. Evidenced by: Translates a technical platform issue into terms a non-engineer decision-maker acts on. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the communication standard other platform leads adopt. Crafts the platform narrative several teams reuse to align stakeholders. Scope: communication across a cross-team domain.</t>
+          <t>Depth: Briefs senior leaders under pressure — facts, impact, options, and a recommendation inside the first two minutes; one-pagers get forwarded unedited. Evidenced by: Gets a skeptical stakeholder to a decision through a well-framed case. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives the platform narrative to executive audiences and wins decisions and funding. Turns a complex platform investment into an exec-level story that lands the budget. Scope: exec communication for a platform sub-org.</t>
+          <t>Depth: Builds and lands investment cases with executive audiences — pre-wired with skeptics, sized in business terms, honest about risk; coaches others for executive rooms and runs the operating reviews an organization communicates through. Evidenced by: Crafts the platform narrative several teams reuse to align stakeholders. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
         <is>
-          <t>Depth: Represents developer productivity and platform value to the top of the company. Sets how the function tells its story to the board and business. Scope: communication across the platform function.</t>
+          <t>Depth: Operates the executive room as a peer — advances positions, absorbs hostile questioning without defensiveness, and changes the room's decision more often than not. Evidenced by: Turns a complex platform investment into an exec-level story that lands the budget. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K37" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide platform narrative. Speaks for platform to the board and externally as a recognized voice. Scope: org-wide and external communication.</t>
+          <t>Depth: Operates the executive room as a peer — advances positions, absorbs hostile questioning without defensiveness, and changes the room's decision more often than not. Evidenced by: Sets how the function tells its story to the board and business. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L37" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Speaks for an organization's technical reality to boards, investors, and press; trusted with the messages that cannot be delegated, and organizational credibility survives the appearances. Evidenced by: Speaks for platform to the board and externally as a recognized voice. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -2844,37 +3030,42 @@
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>Freeman, Strategic Management: A Stakeholder Approach (1984)</t>
+          <t>Aligning leadership and cross-functional stakeholders around product direction and trade-offs.</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds working relationships with the platform's stakeholder teams. Turns a frustrated internal customer into a collaborating partner. Scope: stakeholders for one platform team.</t>
+          <t>Freeman, Strategic Management: A Stakeholder Approach (Pitman, 1984) — platform serves many internal stakeholders with conflicting needs, and managing them is the job</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>Depth: Manages a complex, multi-stakeholder relationship for a critical platform, balancing conflicting needs. Brokers a durable agreement between platform and a demanding consumer team. Scope: stakeholders for a high-stakes platform team.</t>
+          <t>Depth: Manages routine stakeholder relationships and communications with normal review. Evidenced by: Turns a frustrated internal customer into a collaborating partner. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the stakeholder-partnership approach other platform leads adopt. Builds the cross-team partnership model several teams manage relationships through. Scope: stakeholder management across a cross-team domain.</t>
+          <t>Depth: Independently aligns conflicting stakeholders and navigates tense executive conversations. Evidenced by: Brokers a durable agreement between platform and a demanding consumer team. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the stakeholder-governance model a sub-org runs on, from partnership forums to expectation-setting and escalation paths. Realigns a strained sub-org-level partnership with a major consumer org. Scope: partnership across a platform sub-org.</t>
+          <t>Depth: Defines stakeholder-engagement approaches others adopt and brokers the hardest alignment. Evidenced by: Builds the cross-team partnership model several teams manage relationships through. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives the function's key executive and cross-functional partnerships. Sets the partnership approach the function relies on. Scope: partnership across the platform function.</t>
+          <t>Depth: Defines stakeholder-engagement approaches others adopt and brokers the hardest alignment. Evidenced by: Realigns a strained sub-org-level partnership with a major consumer org. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K38" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide model for platform's partnerships. Pioneers a stakeholder approach other functions adopt. Scope: org-wide partnership.</t>
+          <t>Depth: Sets executive-engagement strategy and anticipates leadership concerns before they arise. Evidenced by: Sets the partnership approach the function relies on. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L38" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines exemplary stakeholder management for the discipline and is externally credible on it. Evidenced by: Pioneers a stakeholder approach other functions adopt. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -2901,37 +3092,42 @@
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>Cohen &amp; Bradford, Influence Without Authority (1989); Bungay, The Art of Action (2011)</t>
+          <t>Wins outcomes across organizational seams with no formal mandate — exchange in others' currencies, coalition-building, and earned credibility.</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>Depth: Gets outcomes from teams they do not manage through reciprocity and clarity. Aligns another team to a shared platform goal without authority over them. Scope: influence for one platform team.</t>
+          <t>Cohen &amp; Bradford, Influence Without Authority, 3rd ed. (Wiley, 2017) — platform leaders get outcomes across teams they do not own, through reciprocity and clear intent</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>Depth: Aligns multiple teams around a critical platform direction under real disagreement. Builds cross-team agreement on a contested platform standard. Scope: influence for a high-stakes platform team.</t>
+          <t>Depth: Wins cooperation from adjacent teams by trading in their currencies — timing help, review effort, shared credit — rather than escalating. Evidenced by: Aligns another team to a shared platform goal without authority over them. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the alignment approach other platform leads adopt. Drives alignment across a domain by clear intent, commander's-intent style, rather than escalation. Scope: influence across a cross-team domain.</t>
+          <t>Depth: Secures priority from other teams for an initiative with no borrowed authority; builds the case in the other party's terms and repays visibly. Evidenced by: Builds cross-team agreement on a contested platform standard. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds cross-org alignment a sub-org depends on, aligning peer orgs to platform direction. Wins peer-org buy-in for a sub-org-wide platform initiative. Scope: influence across a platform sub-org.</t>
+          <t>Depth: Moves a multi-team domain to a shared position with no mandate — assembles the coalition, converts the best-argued skeptic — and the position holds after they stop pushing. Evidenced by: Drives alignment across a domain by clear intent, commander's-intent style, rather than escalation. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives alignment across the function's peer organizations at the leadership level. Sets the alignment mechanisms the function relies on to move the wider org. Scope: influence across the platform function.</t>
+          <t>Depth: Moves a multi-team domain to a shared position with no mandate — assembles the coalition, converts the best-argued skeptic — and the position holds after they stop pushing. Evidenced by: Wins peer-org buy-in for a sub-org-wide platform initiative. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K39" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets org-wide alignment on platform direction. Pioneers an influence model that aligns the whole company behind platform bets. Scope: org-wide influence.</t>
+          <t>Depth: Shifts organization-level outcomes through people several seams away who advocate the position as their own; lands decisions while holding a minority of the formal power in the room. Evidenced by: Sets the alignment mechanisms the function relies on to move the wider org. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L39" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Shapes industry and market context in the organization's favor — standards bodies, open ecosystems, talent narratives — so external forces push where the organization wants to go. Evidenced by: Pioneers an influence model that aligns the whole company behind platform bets. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -2958,37 +3154,42 @@
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>Grove, High Output Management (1983); Drucker (1967)</t>
+          <t>Spends leadership time where it multiplies — deliberate calendar design, high-leverage intervention choice, and systematic abandonment of low-value work.</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>Depth: Spends their own time on the few activities that most move the team, and audits where it actually goes. Drops a low-leverage habit such as reviewing every change themselves once they see its cost. Scope: personal leverage on one platform team.</t>
+          <t>Grove, High Output Management (Random House, 1983) — a manager's output is the leveraged output of everyone they touch, and time is the one non-renewable resource</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>Depth: Redesigns their week around the highest-leverage work on a high-stakes team — the decisions, unblocks, and reviews only they can do — and hands off the rest. Restructures how they spend time so a critical platform team stops waiting on them. Scope: personal leverage on a critical platform team.</t>
+          <t>Depth: Runs a deliberate calendar that matches stated priorities — protected one-on-ones, deep work, and team time; declines low-leverage meetings with alternatives offered. Evidenced by: Drops a low-leverage habit such as reviewing every change themselves once they see its cost. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the leverage practice other platform leads pick up, favoring mechanisms that multiply reach over adding meetings. Publishes an operating cadence several leads adopt to reclaim their own high-leverage time. Scope: leverage practice across a cross-team domain.</t>
+          <t>Depth: Prunes their own involvement ruthlessly as complexity grows — automates, delegates, or kills recurring work every quarter — and models sustainable pace through crunch. Evidenced by: Restructures how they spend time so a critical platform team stops waiting on them. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the operating rhythm a platform sub-org runs on so decisions happen at the lowest capable level rather than on one desk. Removes themselves as a bottleneck across the sub-org by installing the mechanisms that decide without them. Scope: leverage across a platform sub-org.</t>
+          <t>Depth: Chooses interventions by multiplier across many teams — the review that shapes ten decisions, the document that aligns three roadmaps — declining the rest by policy; audits their time and publishes the changes. Evidenced by: Publishes an operating cadence several leads adopt to reclaim their own high-leverage time. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives how the function protects its leaders' focus and concentrates effort on the few bets that matter. Sets the focus and leverage norms leaders across the function organize their time around. Scope: leverage across the platform function.</t>
+          <t>Depth: Chooses interventions by multiplier across many teams — the review that shapes ten decisions, the document that aligns three roadmaps — declining the rest by policy; audits their time and publishes the changes. Evidenced by: Removes themselves as a bottleneck across the sub-org by installing the mechanisms that decide without them. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K40" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide expectation for how platform leadership spends its scarce attention. Pioneers a leverage model peer functions adopt. Scope: org-wide leadership leverage.</t>
+          <t>Depth: Allocates attention like a portfolio at organizational scale — deep on the few places they are the unique unlock, delegated on the rest — and says which is which out loud. Evidenced by: Sets the focus and leverage norms leaders across the function organize their time around. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L40" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Spends presence deliberately as an organizational signal — where they show up moves priorities — and guards the organization's focus by limiting concurrent top priorities and abandoning stale initiatives by name. Evidenced by: Pioneers a leverage model peer functions adopt. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -3015,37 +3216,42 @@
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>Marquet, Turn the Ship Around! (2012)</t>
+          <t>Hands over whole outcomes with context and calibrated support, pushes decision rights to where the information lives, and builds organizations that run on intent rather than presence.</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>Depth: Delegates real ownership, not just tasks, and matches each handoff to the engineer's readiness. Hands a platform workstream to an engineer with the decision rights to run it, then holds back. Scope: delegation on one platform team.</t>
+          <t>Marquet, Turn the Ship Around!: A True Story of Turning Followers into Leaders (Portfolio/Penguin, 2013; orig. 2012) — leadership scales by pushing authority to where the information is, creating leaders rather than followers</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>Depth: Empowers senior engineers and leads to own hard, ambiguous platform work and make the calls themselves. Grows a report into someone who runs a critical workstream end to end without checking in. Scope: delegation on a critical platform team.</t>
+          <t>Depth: Delegates whole outcomes with context and check-in contracts matched to each person's readiness — and resists snatching work back when it wobbles. Evidenced by: Hands a platform workstream to an engineer with the decision rights to run it, then holds back. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the delegation and empowerment standard other platform leads adopt, favoring intent and guardrails over instructions. Gets outcomes across a domain by stating clear intent and letting other leaders decide how. Scope: empowerment across a cross-team domain.</t>
+          <t>Depth: Hands ownership of critical, visible work to someone not yet proven and scaffolds them to success, letting them keep the credit; the team runs a week without them and nothing stalls. Evidenced by: Grows a report into someone who runs a critical workstream end to end without checking in. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the decision-rights model a platform sub-org runs on so authority sits with the people closest to the work. Pushes a class of decisions down to team leaders across the sub-org and stops being consulted on them. Scope: empowerment across a platform sub-org.</t>
+          <t>Depth: Pushes decisions down across multiple teams — publishes decision rights so teams stop escalating what they can decide themselves; involvement is exception-based, and everyone knows which is which. Evidenced by: Gets outcomes across a domain by stating clear intent and letting other leaders decide how. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives how the function distributes authority, growing decision-makers rather than approvers. Sets the empowerment norms leaders across the function lead by. Scope: empowerment across the platform function.</t>
+          <t>Depth: Pushes decisions down across multiple teams — publishes decision rights so teams stop escalating what they can decide themselves; involvement is exception-based, and everyone knows which is which. Evidenced by: Pushes a class of decisions down to team leaders across the sub-org and stops being consulted on them. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K41" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide expectation that platform leadership creates leaders, not dependence. Pioneers a decision-rights model other functions adopt. Scope: org-wide empowerment.</t>
+          <t>Depth: Builds organizations that run on mechanisms rather than presence — delegated authorities with audit trails, pre-declared tripwires — and grants leaders consequential authority held to outcomes, not methods. Evidenced by: Sets the empowerment norms leaders across the function lead by. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L41" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Runs an organization on intent — direction and guardrails clear enough that leaders act correctly without asking — and treats every upward escalation as a design flaw to fix. Evidenced by: Pioneers a decision-rights model other functions adopt. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -3072,37 +3278,42 @@
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>Eurich, Insight (2017); Lombardo &amp; Eichinger (2000)</t>
+          <t>Seeks external feedback on their own behavior, knows their failure patterns, and extracts lessons from first-time situations fast enough to lead credibly in them.</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>Depth: Seeks feedback on their own leadership and acts on it visibly. Changes a specific behavior after hearing it lands badly, rather than defending it. Scope: personal growth on one platform team.</t>
+          <t>Eurich, What Self-Awareness Really Is (and How to Cultivate It), Harvard Business Review (2018) — accurate self-knowledge and the ability to learn from new experience predict leadership growth</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>Depth: Reads their own impact on a high-stakes team accurately and adapts to unfamiliar problems quickly. Names a blind spot and adjusts before it costs the team, using an outside read to check their own. Scope: self-awareness on a critical platform team.</t>
+          <t>Depth: Asks for feedback on their own practice and changes visibly in response — "you said X, I changed Y" — keeping a running list of their own failure patterns. Evidenced by: Changes a specific behavior after hearing it lands badly, rather than defending it. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the norm that platform leads solicit and act on feedback, and models learning in the open. Runs feedback mechanisms several leads adopt to see their own effect on others. Scope: learning culture across a cross-team domain.</t>
+          <t>Depth: Knows their failure modes under pressure and manages them in the moment; staffs deliberately against known weaknesses and seeks disconfirming input before hard calls. Evidenced by: Names a blind spot and adjusts before it costs the team, using an outside read to check their own. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the leadership-feedback and development practice a sub-org relies on to keep its leaders self-correcting. Turns a leader's blind spot around across the sub-org by making honest upward feedback safe and routine. Scope: leader growth across a platform sub-org.</t>
+          <t>Depth: Runs structured input on themselves — 360s, skip-level themes — and closes the loop publicly on what changed; retools openly for first-time challenges so others copy the learning method. Evidenced by: Runs feedback mechanisms several leads adopt to see their own effect on others. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives how the function grows self-aware, adaptable leaders as the technology and org shift. Sets the learning-agility expectations leaders across the function are developed against. Scope: leadership growth across the platform function.</t>
+          <t>Depth: Runs structured input on themselves — 360s, skip-level themes — and closes the loop publicly on what changed; retools openly for first-time challenges so others copy the learning method. Evidenced by: Turns a leader's blind spot around across the sub-org by making honest upward feedback safe and routine. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K42" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide expectation that platform leadership learns and adapts in the open. Pioneers a leadership-development model peer functions adopt. Scope: org-wide leadership learning.</t>
+          <t>Depth: Compensates deliberately for the seniority feedback vacuum — cultivates truth-tellers, rewards bearers of unwelcome news about themselves, and retires their own outdated playbook when the organization outgrows it. Evidenced by: Sets the learning-agility expectations leaders across the function are developed against. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L42" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Institutionalizes challenge to their own judgment — red teams, protected dissent — and manages how their moods and offhand comments get amplified across an organization. Evidenced by: Pioneers a leadership-development model peer functions adopt. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -3129,37 +3340,42 @@
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>Loehr &amp; Schwartz, The Power of Full Engagement (2003)</t>
+          <t>Sustains effectiveness under prolonged pressure, recovers from setbacks, and designs sustainable pace into how teams operate rather than modeling heroics.</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>Depth: Keeps themselves and the team steady through incidents and crunch without burning out. Protects the team's sustainable pace during an on-call-heavy stretch instead of normalizing heroics. Scope: resilience on one platform team.</t>
+          <t>Loehr &amp; Schwartz, The Power of Full Engagement: Managing Energy, Not Time, Is the Key to High Performance and Personal Renewal (Free Press, 2003) — performance is a function of managed energy, not time, and sustainable pace beats heroics</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>Depth: Holds their composure and the team's under sustained operational pressure on a critical platform. Absorbs the stress of a severe outage period and keeps the team functioning rather than fraying. Scope: resilience on a critical platform team.</t>
+          <t>Depth: Stays effective and steady under pressure — recovers from setbacks, manages their own energy, and models a sustainable pace others learn from watching. Evidenced by: Protects the team's sustainable pace during an on-call-heavy stretch instead of normalizing heroics. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the sustainable-pace norms other platform leads adopt, treating on-call and toil load as a health metric. Acts on a burnout signal across the domain before it becomes attrition, changing the load rather than the people. Scope: sustainable pace across a cross-team domain.</t>
+          <t>Depth: Holds up through prolonged pressure — incident sieges, crunch, organizational turbulence — helping the team stay resilient and refusing burnout-driven decisions. Evidenced by: Absorbs the stress of a severe outage period and keeps the team functioning rather than fraying. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the operating norms a platform sub-org uses to keep pace sustainable through scaling and incidents. Reshapes on-call and workload across the sub-org so resilience does not depend on individual heroics. Scope: sustainable pace across a platform sub-org.</t>
+          <t>Depth: Builds resilience into how multiple teams operate — on-call health, recovery after pushes, load balancing — and repairs burnout risk at scale. Evidenced by: Acts on a burnout signal across the domain before it becomes attrition, changing the load rather than the people. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives how the function sustains its people through the always-on nature of platform work. Sets the sustainable-pace expectations leaders across the function are held to. Scope: resilience across the platform function.</t>
+          <t>Depth: Builds resilience into how multiple teams operate — on-call health, recovery after pushes, load balancing — and repairs burnout risk at scale. Evidenced by: Reshapes on-call and workload across the sub-org so resilience does not depend on individual heroics. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K43" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide expectation that platform delivers durably, not through burnout. Pioneers a sustainable-operations model peer functions adopt. Scope: org-wide sustainable pace.</t>
+          <t>Depth: Stewards organizational resilience — capacity buffers, crisis rotation, energy management for senior leaders — and holds the line when business pressure argues for permanent crunch. Evidenced by: Sets the sustainable-pace expectations leaders across the function are held to. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L43" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Shapes a resilient, sustainable culture across an organization; the organization absorbs shocks without breaking people, and the practice is referenced beyond it. Evidenced by: Pioneers a sustainable-operations model peer functions adopt. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -3186,37 +3402,42 @@
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>Kahneman, Thinking, Fast and Slow (2011)</t>
+          <t>Makes sound calls with incomplete information.</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>Depth: Makes timely calls with incomplete information and states the assumptions behind them. Makes a reversible platform decision quickly rather than stalling for certainty that will not come. Scope: decisions on one platform team.</t>
+          <t>Kahneman, Thinking, Fast and Slow (Farrar, Straus and Giroux, 2011) — sound decisions require guarding against bias and calibrating confidence to the evidence</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>Depth: Makes high-stakes, hard-to-reverse calls on a critical platform and guards against their own bias. Frames a one-way-door platform decision explicitly and gathers the evidence its weight warrants. Scope: decisions on a critical platform team.</t>
+          <t>Depth: Decides independently within their components; evaluates alternatives honestly. Evidenced by: Makes a reversible platform decision quickly rather than stalling for certainty that will not come. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the decision-making discipline other platform leads adopt, with clear owners, reversibility tests, and recorded rationale. Installs a decision framework several teams now use to make calls under ambiguity. Scope: decision quality across a cross-team domain.</t>
+          <t>Depth: Makes architectural choices for a domain that hold up over months. Evidenced by: Frames a one-way-door platform decision explicitly and gathers the evidence its weight warrants. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the decision-rights and judgment norms a sub-org runs on so hard calls get made well and fast across it. Raises the quality of consequential decisions across the sub-org by making the reasoning and the owner explicit. Scope: decision-making across a platform sub-org.</t>
+          <t>Depth: Foresees second-order consequences; sets decision frameworks for teams. Evidenced by: Installs a decision framework several teams now use to make calls under ambiguity. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J44" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives how the function makes irreversible, high-ambiguity bets and lives with the trade-offs. Sets the decision standard leaders across the function are calibrated to. Scope: decision-making across the platform function.</t>
+          <t>Depth: Foresees second-order consequences; sets decision frameworks for teams. Evidenced by: Raises the quality of consequential decisions across the sub-org by making the reasoning and the owner explicit. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K44" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide expectation for how platform leadership decides under uncertainty. Pioneers a decision model peer functions adopt. Scope: org-wide decision-making.</t>
+          <t>Depth: Sets decision-making frameworks for the org. Evidenced by: Sets the decision standard leaders across the function are calibrated to. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L44" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Visionary judgment; sees structural causes others miss. Evidenced by: Pioneers a decision model peer functions adopt. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -3243,37 +3464,42 @@
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>Mayer, Davis &amp; Schoorman (1995); ACM Code of Ethics (2018)</t>
+          <t>Earns and keeps trust through consistency and courage — keeping commitments, telling unwelcome truths, and holding the ethical line when it is costly.</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>Depth: Acts consistently and honestly, keeps commitments, and is straight about mistakes. Makes the honest call on a platform reliability or security risk even when it is inconvenient to admit. Scope: trust on one platform team.</t>
+          <t>Mayer, Davis &amp; Schoorman, An Integrative Model of Organizational Trust, Academy of Management Review 20(3), 709-734 (1995) — trust is built on ability, benevolence, and integrity, and platform leaders hold outsized access and impact</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
-          <t>Depth: Holds the ethical line on a critical platform where access, data, and reliability carry real stakes. Refuses a shortcut that would trade user trust or safety for speed, and says why. Scope: integrity on a critical platform team.</t>
+          <t>Depth: Makes the unpopular-but-right call under pressure and absorbs the cost personally; protects the person who raised the flag and handles sensitive information impeccably. Evidenced by: Makes the honest call on a platform reliability or security risk even when it is inconvenient to admit. Scope: one platform team.</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the ethical and trust norms other platform leads adopt around access, data, and honest incident disclosure. Establishes the do-the-right-thing expectations several teams now hold each other to. Scope: integrity across a cross-team domain.</t>
+          <t>Depth: Makes the unpopular-but-right call under pressure and absorbs the cost personally; protects the person who raised the flag and handles sensitive information impeccably. Evidenced by: Refuses a shortcut that would trade user trust or safety for speed, and says why. Scope: a complex / critical platform team.</t>
         </is>
       </c>
       <c r="I45" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the trust and integrity expectations a platform sub-org operates by, from privileged-access ethics to honest reporting. Makes candid, blameless honesty the norm across the sub-org even when the news is bad. Scope: integrity across a platform sub-org.</t>
+          <t>Depth: Serves as the honest broker across teams — disputing parties accept their account of the facts — and carries uncomfortable systemic truths to the room that can fix them. Evidenced by: Establishes the do-the-right-thing expectations several teams now hold each other to. Scope: a platform domain (cross-team).</t>
         </is>
       </c>
       <c r="J45" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives the function's ethical posture on the outsized access and impact platform holds. Sets the integrity standard leaders across the function are trusted to uphold. Scope: ethics across the platform function.</t>
+          <t>Depth: Serves as the honest broker across teams — disputing parties accept their account of the facts — and carries uncomfortable systemic truths to the room that can fix them. Evidenced by: Makes candid, blameless honesty the norm across the sub-org even when the news is bad. Scope: a platform sub-org.</t>
         </is>
       </c>
       <c r="K45" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide expectation for how platform leadership stewards trust, access, and impact. Pioneers an ethics model peer functions and the wider field reference. Scope: org-wide integrity and trust.</t>
+          <t>Depth: Builds mechanisms that make integrity cheap at scale — ethics review in design, safe escalation with follow-through, fairness systems whose losers affirm the process — and stops launches on ethical grounds with the business case for trust. Evidenced by: Sets the integrity standard leaders across the function are trusted to uphold. Scope: the platform function.</t>
+        </is>
+      </c>
+      <c r="L45" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Holds an organization's line when the profitable path and the right path diverge — the hard disclosure, the walked-away revenue — and those moments become the story the culture tells about itself. Evidenced by: Pioneers an ethics model peer functions and the wider field reference. Scope: org-wide platform.</t>
         </is>
       </c>
     </row>
@@ -5433,326 +5659,1460 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A45"/>
+  <dimension ref="A1:D97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="110" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Sources</t>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Grounds</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Link</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>**Schmidt &amp; Hunter, selection-methods meta-analysis (1998)** — Hiring &amp; selection.</t>
-        </is>
-      </c>
+          <t>Meta-analysis of 85 years of selection-method validity; grounds structured, evidence-based hiring judgment</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Schmidt &amp; Hunter, The Validity and Utility of Selection Methods in Personnel Psychology, Psychological Bulletin 124(2), 262-274 (1998)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Hiring &amp; selection</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>**Tuckman, Developmental Sequence in Small Groups (1965)** — Onboarding &amp; team formation.</t>
+          <t>Forming-storming-norming-performing team stages</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Tuckman, Developmental Sequence in Small Groups, Psychological Bulletin 63(6), 384-399 (1965)</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Onboarding &amp; team formation</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1037/h0022100</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>**Whitmore, Coaching for Performance (1992); Google Project Oxygen** — Coaching &amp; development.</t>
+          <t>GROW model; origin of the coach-not-tell manager stance</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Whitmore, Coaching for Performance: GROWing Human Potential and Purpose, 4th ed. (Nicholas Brealey, 2009; orig. 1992)</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Coaching &amp; development</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>https://www.nicholasbrealey.com/coaching-for-performance/</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>**Hewlett, Forget a Mentor, Find a Sponsor (2013)** — Career development &amp; sponsorship.</t>
+          <t>Distinguishes sponsorship (advocacy, reputational risk) from mentorship (advice)</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Hewlett, Forget a Mentor, Find a Sponsor: The New Way to Fast-Track Your Career (Harvard Business Review Press, 2013)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Career development &amp; sponsorship</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>https://www.barnesandnoble.com/w/forget-a-mentor-find-a-sponsor-sylvia-ann-hewlett/1114264520</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>**Grove, High Output Management (1983)** — Performance management.</t>
+          <t>Origin of management-by-objectives cascading goal-setting that OKRs formalize</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Grove, High Output Management (Random House, 1983)</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Performance management</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>https://www.penguinrandomhouse.com/books/163289/high-output-management-by-andrew-s-grove/</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>**Edmondson, The Fearless Organization (2018); Project Aristotle** — Psychological safety &amp; team health.</t>
+          <t>Practitioner-facing extension of Edmondson's 1999 psychological-safety research to team leadership practice</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Edmondson, The Fearless Organization: Creating Psychological Safety in the Workplace for Learning, Innovation, and Growth (Wiley, 2018)</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Psychological safety &amp; team health</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>https://www.wiley.com/en-us/The+Fearless+Organization%3A+Creating+Psychological+Safety+in+the+Workplace+for+Learning%2C+Innovation%2C+and+Growth-p-9781119477242</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>**Deci &amp; Ryan, Self-Determination Theory (2000); Herzberg (1968)** — Motivation, engagement &amp; retention.</t>
+          <t>Autonomy, competence, relatedness drive durable engagement over extrinsic reward</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Deci &amp; Ryan, The "What" and "Why" of Goal Pursuits: Human Needs and the Self-Determination of Behavior, Psychological Inquiry 11(4), 227-268 (2000)</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Motivation, engagement &amp; retention</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1207/S15327965PLI1104_01</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>**Perri, Escaping the Build Trap (2018); Skelton &amp; Pais, Team Topologies (2019)** — Platform vision &amp; roadmap.</t>
+          <t>Org-level product strategy vs. output-shipping; grounds strategic/commercial leveling</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Perri, Escaping the Build Trap: How Effective Product Management Creates Real Value (O'Reilly, 2018)</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Platform vision &amp; roadmap</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.oreilly.com/library/view/escaping-the-build/9781491973783/</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>**Noda, Storey, Forsgren &amp; Greiler, DevEx: What Actually Drives Productivity (ACM Queue, 2023)** — Internal user research &amp; discovery.</t>
+          <t>Feedback loops, cognitive load, flow state as the measurable drivers of developer productivity</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Noda, Storey, Forsgren &amp; Greiler, DevEx: What Actually Drives Productivity, ACM Queue 21(2) (2023)</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Internal user research &amp; discovery</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>https://queue.acm.org/detail.cfm?id=3595878</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>**Cagan, Inspired (2008)** — Platform value &amp; business case.</t>
+          <t>SVPG discovery-risk framework (value/usability/feasibility/viability); PM domain-expertise and discovery-judgment anchor</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Cagan, INSPIRED: How to Create Tech Products Customers Love, 2nd Edition (Wiley, 2018)</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Platform value &amp; business case</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>https://www.svpg.com/inspired-2nd-edition/</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>**Spotify Engineering, How We Use Golden Paths (2020)** — Golden paths &amp; paved roads.</t>
+          <t>Origin of the golden-path/paved-road pattern for internal platforms</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Spotify Engineering, How We Use Golden Paths to Solve Fragmentation in Our Software Ecosystem (Spotify Engineering Blog, 2020)</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Golden paths &amp; paved roads</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>https://engineering.atspotify.com/2020/08/how-we-use-golden-paths-to-solve-fragmentation-in-our-software-ecosystem/</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>**Bottcher, What I Talk About When I Talk About Platforms (martinfowler.com, 2018)** — Self-service &amp; platform interfaces.</t>
+          <t>Thinnest-viable-platform framing; a platform's job is to cut cognitive load through self-service interfaces</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Bottcher, What I Talk About When I Talk About Platforms (martinfowler.com, 2018)</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Self-service &amp; platform interfaces</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>https://martinfowler.com/articles/talk-about-platforms.html</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>**Winters, Manshreck &amp; Wright, Software Engineering at Google (2020) - deprecation chapter** — Adoption &amp; migration strategy.</t>
+          <t>Distinguishes programming from org-scale software engineering; anchors org-wide standard-setting levels</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Winters, Manshreck &amp; Wright, Software Engineering at Google: Lessons Learned from Programming Over Time (O'Reilly, 2020)</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Adoption &amp; migration strategy</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>https://abseil.io/resources/swe-book</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>**CNCF TAG App Delivery, Platform Engineering Maturity Model (2023)** — Platform advocacy &amp; enablement.</t>
+          <t>Maturity tiers for platform-as-a-product investment across people/process/policy/technology; link verified 200</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>CNCF TAG App Delivery, Platform Engineering Maturity Model (2023)</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Platform advocacy &amp; enablement</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>https://tag-app-delivery.cncf.io/whitepapers/platform-eng-maturity-model/</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>**Beyer, Jones, Petoff &amp; Murphy, Site Reliability Engineering (2016)** — Reliability, SLOs &amp; error budgets.</t>
+          <t>Google's published postmortem/root-cause and diagnostic-tooling practice; anchors debugging leveling</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Beyer, Jones, Petoff &amp; Murphy (eds.), Site Reliability Engineering: How Google Runs Production Systems (O'Reilly/Google, 2016)</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Reliability, SLOs &amp; error budgets</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>https://sre.google/sre-book/table-of-contents/</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>**PagerDuty, Incident Response Guide (2017); Allspaw, Blameless PostMortems (2012)** — Incident &amp; operational-risk leadership.</t>
+          <t>Named incident-command roles severity classification and on-call rotation design practice guide</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>PagerDuty, Incident Response Documentation (accessed 2026-07)</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Incident &amp; operational-risk leadership</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>https://response.pagerduty.com/</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>**Majors, Fong-Jones &amp; Miranda, Observability Engineering (2022)** — Observability &amp; health signals.</t>
+          <t>High-cardinality, high-dimensionality telemetry vs. traditional monitoring</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Majors, Fong-Jones &amp; Miranda, Observability Engineering: Achieving Production Excellence (O'Reilly, 2022)</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Observability &amp; health signals</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>https://www.oreilly.com/library/view/observability-engineering/9781492076438/</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>**Beyer, Jones, Petoff &amp; Murphy, Site Reliability Engineering (2016) - toil chapter** — Toil reduction &amp; automation.</t>
+          <t>USE method and capacity/performance methodology coupling cost, capacity and performance</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Gregg, Systems Performance: Enterprise and the Cloud, 2nd ed. (Addison-Wesley, 2020)</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Capacity, performance &amp; cost</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>https://www.brendangregg.com/systems-performance-2nd-edition-book.html</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>**Gregg, Systems Performance (2nd ed., 2020)** — Capacity, performance &amp; cost.</t>
+          <t>Conway's Law: system design mirrors the communication structure of the organization that builds it</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Conway, How Do Committees Invent?, Datamation 14(4), 28-31 (1968)</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Platform architecture stewardship</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>https://www.melconway.com/Home/Committees_Paper.html</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>**Conway (1968); Nygard, Documenting Architecture Decisions (2011)** — Platform architecture stewardship.</t>
+          <t>Deployment pipeline environment-parity and release-automation discipline</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Humble &amp; Farley, Continuous Delivery: Reliable Software Releases through Build Test and Deployment Automation (Addison-Wesley, 2010)</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Engineering standards &amp; quality</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>https://continuousdelivery.com/</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>**Humble &amp; Farley, Continuous Delivery (2010)** — Engineering standards &amp; quality.</t>
+          <t>Origin of the technical-debt metaphor (principal and accruing interest)</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Cunningham, The WyCash Portfolio Management System, OOPSLA 1992 Experience Report</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Technical debt &amp; modernization</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>https://c2.com/doc/oopsla92.html</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>**Cunningham, The WyCash Portfolio Management System (1992)** — Technical debt &amp; modernization.</t>
+          <t>Sizing teams, technical strategy, and org design for engineering leadership</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Larson, An Elegant Puzzle: Systems of Engineering Management (Stripe Press, 2019)</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Technical strategy &amp; investment</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>https://press.stripe.com/an-elegant-puzzle</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>**Larson, An Elegant Puzzle (2019); Wardley Maps (2016)** — Technical strategy &amp; investment.</t>
+          <t>38-competency leadership model incl. Financial Acumen; industry-standard leveling reference</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Korn Ferry, Korn Ferry Leadership Architect Global Competency Framework (2014)</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Vendor &amp; build/buy/adopt strategy</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>https://www.kornferry.com/capabilities/talent-suite/korn-ferry-assess/leadership-architect</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>**Korn Ferry Leadership Architect (2014) - Financial Acumen** — Vendor &amp; build/buy/adopt strategy.</t>
+          <t>Tiered verification levels (L1 baseline through L3 advanced) for defense-in-depth security controls</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>OWASP Foundation, OWASP Application Security Verification Standard (accessed 2026-07)</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Secure-by-default platform &amp; guardrails</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>https://owasp.org/www-project-application-security-verification-standard/</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>**OWASP, Application Security Verification Standard (v4, 2019)** — Secure-by-default platform &amp; guardrails.</t>
+          <t>Estimation as a probabilistic forecast to calibrate, distinct from Code Complete</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>McConnell, Software Estimation: Demystifying the Black Art (Microsoft Press, 2006)</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Planning &amp; estimation</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>https://www.construx.com/store/software-estimation-demystifying-the-black-art/</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>**McConnell, Software Estimation (2006)** — Planning &amp; estimation.</t>
-        </is>
-      </c>
+          <t>Cost-of-delay and queueing-theory economics for prioritization decisions; verified via web search</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Reinertsen, The Principles of Product Development Flow: Second Generation Lean Product Development (Celeritas, 2009)</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Prioritization &amp; trade-offs</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>**Reinertsen, The Principles of Product Development Flow (2009)** — Prioritization &amp; trade-offs.</t>
+          <t>Adding manpower to a late project makes it later; coordination cost scales with headcount</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Brooks, The Mythical Man-Month: Essays on Software Engineering, Anniversary ed. (Addison-Wesley, 1995; orig. 1975)</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Capacity &amp; resource allocation</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/The_Mythical_Man-Month</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>**Brooks, The Mythical Man-Month (1975)** — Capacity &amp; resource allocation.</t>
+          <t>Empirical linkage between deployment/release engineering maturity and organizational performance</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Forsgren, Humble &amp; Kim, Accelerate: The Science of Lean Software and DevOps (IT Revolution Press, 2018)</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Predictable delivery &amp; flow</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>https://itrevolution.com/product/accelerate/</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>**Forsgren, Humble &amp; Kim, Accelerate (2018)** — Predictable delivery &amp; flow.</t>
-        </is>
-      </c>
+          <t>14 points for management; continuous, systemic process improvement over inspection</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Deming, Out of the Crisis (MIT Center for Advanced Engineering Study, 1986)</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Process &amp; continuous improvement</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>**Forsgren, Humble &amp; Kim, Accelerate (2018) - DORA four keys; SPACE (2021)** — Engineering metrics &amp; delivery health.</t>
+          <t>Six-function (incl. Govern) taxonomy for organizing enterprise cybersecurity risk strategy</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>NIST, The NIST Cybersecurity Framework (CSF) 2.0, NIST CSWP 29 (2024)</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Dependency &amp; risk management</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>https://csrc.nist.gov/pubs/cswp/29/the-nist-cybersecurity-framework-csf-20/final</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>**Deming, Out of the Crisis (1986)** — Process &amp; continuous improvement.</t>
+          <t>Strategy kernel (diagnosis, guiding policy, coherent action) as the test for real vs. bad strategy</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Rumelt, Good Strategy Bad Strategy: The Difference and Why It Matters (Crown Business, 2011)</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Strategy formulation</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>https://www.penguinrandomhouse.com/books/198888/good-strategy-bad-strategy-by-richard-p-rumelt/</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>**NIST Cybersecurity Framework (2014); PMI PMBOK (2021)** — Dependency &amp; risk management.</t>
+          <t>Eight-step model for leading organizational change through to durable adoption</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Kotter, Leading Change (Harvard Business School Press, 1996)</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Leading change &amp; transformation</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>https://openlibrary.org/books/OL982607M/Leading_Change</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>**Rumelt, Good Strategy Bad Strategy (2011)** — Strategy formulation.</t>
-        </is>
-      </c>
+          <t>Team boundaries; org-level team formation patterns</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Skelton &amp; Pais, Team Topologies (IT Revolution, 2019)</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Organizational &amp; team design</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>**Kotter, Leading Change (1996)** — Leading change &amp; transformation.</t>
+          <t>Structuring executive communication around audience needs, not speaker content</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Duarte, HBR Guide to Persuasive Presentations (Harvard Business Review Press, 2012)</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Executive &amp; stakeholder communication</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>https://store.hbr.org/product/hbr-guide-to-persuasive-presentations/10058</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>**Skelton &amp; Pais, Team Topologies (2019); Conway (1968)** — Organizational &amp; team design.</t>
-        </is>
-      </c>
+          <t>Origin of stakeholder theory: managing for groups who affect or are affected by the organization</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>Freeman, Strategic Management: A Stakeholder Approach (Pitman, 1984)</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Stakeholder management &amp; partnership</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>**Duarte, HBR Guide to Persuasive Presentations (2012)** — Executive &amp; stakeholder communication.</t>
+          <t>Exchange Model of influence: trading in others' currencies absent formal authority</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Cohen &amp; Bradford, Influence Without Authority, 3rd ed. (Wiley, 2017)</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Cross-org influence &amp; alignment</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>https://www.wiley.com/en-us/Influence+Without+Authority,+3rd+Edition-p-9781119347712</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>**Freeman, Strategic Management: A Stakeholder Approach (1984)** — Stakeholder management &amp; partnership.</t>
-        </is>
-      </c>
+          <t>Leader-leader model: pushing authority and decision rights down to where the information is</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Marquet, Turn the Ship Around!: A True Story of Turning Followers into Leaders (Portfolio/Penguin, 2013; orig. 2012)</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Delegation &amp; empowerment</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>**Cohen &amp; Bradford, Influence Without Authority (1989); Bungay, The Art of Action (2011)** — Cross-org influence &amp; alignment.</t>
+          <t>Internal/external self-awareness distinction; feedback-seeking research across ~5,000 participants</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Eurich, What Self-Awareness Really Is (and How to Cultivate It), Harvard Business Review (2018)</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Self-awareness &amp; learning agility</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>https://hbr.org/2018/01/what-self-awareness-really-is-and-how-to-cultivate-it</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>**Grove, High Output Management (1983); Drucker (1967)** — Managerial leverage &amp; focus.</t>
-        </is>
-      </c>
+          <t>Sustainable performance managed through energy (physical, emotional, mental, spiritual), not just time</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Loehr &amp; Schwartz, The Power of Full Engagement: Managing Energy, Not Time, Is the Key to High Performance and Personal Renewal (Free Press, 2003)</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>Resilience &amp; sustainable pace</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>**Marquet, Turn the Ship Around! (2012)** — Delegation &amp; empowerment.</t>
+          <t>System 1 / System 2 reasoning; basis for structured decision-making under uncertainty</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Kahneman, Thinking, Fast and Slow (Farrar, Straus and Giroux, 2011)</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Decision-making under uncertainty</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Thinking,_Fast_and_Slow</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>**Eurich, Insight (2017); Lombardo &amp; Eichinger (2000)** — Self-awareness &amp; learning agility.</t>
+          <t>Ability/benevolence/integrity model of trustworthiness; foundational organizational-trust theory</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Mayer, Davis &amp; Schoorman, An Integrative Model of Organizational Trust, Academy of Management Review 20(3), 709-734 (1995)</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Ethics, integrity &amp; trust</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>https://people.wku.edu/richard.miller/Mayer%20Trust%20article.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="4" t="inlineStr">
-        <is>
-          <t>**Loehr &amp; Schwartz, The Power of Full Engagement (2003)** — Resilience &amp; sustainable pace.</t>
-        </is>
-      </c>
+      <c r="A43" s="4" t="inlineStr"/>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Schmidt &amp; Hunter, The Validity and Utility of Selection Methods in Personnel Psychology, Psychological Bulletin 124(2), 262-274 (1998)</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr"/>
+      <c r="D43" s="4" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>**Kahneman, Thinking, Fast and Slow (2011)** — Decision-making under uncertainty.</t>
-        </is>
-      </c>
+      <c r="A44" s="4" t="inlineStr"/>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>GitLab Handbook, Engineering Management Job Framework (accessed 2026-07) — https://handbook.gitlab.com/job-families/engineering/engineering-management/</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr"/>
+      <c r="D44" s="4" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="4" t="inlineStr">
-        <is>
-          <t>**Mayer, Davis &amp; Schoorman (1995); ACM Code of Ethics (2018)** — Ethics, integrity &amp; trust.</t>
-        </is>
-      </c>
+      <c r="A45" s="4" t="inlineStr"/>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>Tuckman, Developmental Sequence in Small Groups, Psychological Bulletin 63(6), 384-399 (1965) — https://doi.org/10.1037/h0022100</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr"/>
+      <c r="D45" s="4" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr"/>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>Whitmore, Coaching for Performance: GROWing Human Potential and Purpose, 4th ed. (Nicholas Brealey, 2009; orig. 1992) — https://www.nicholasbrealey.com/coaching-for-performance/</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr"/>
+      <c r="D46" s="4" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr"/>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>Google re:Work, Following the Data: The Research Behind Great Managers (Project Oxygen research, accessed 2026-07) — https://rework.withgoogle.com/intl/en/guides/following-the-data-the-research-behind-great-managers</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr"/>
+      <c r="D47" s="4" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr"/>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>Hewlett, Forget a Mentor, Find a Sponsor: The New Way to Fast-Track Your Career (Harvard Business Review Press, 2013) — https://www.barnesandnoble.com/w/forget-a-mentor-find-a-sponsor-sylvia-ann-hewlett/1114264520</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr"/>
+      <c r="D48" s="4" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr"/>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>Grove, High Output Management (Random House, 1983) — https://www.penguinrandomhouse.com/books/163289/high-output-management-by-andrew-s-grove/</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr"/>
+      <c r="D49" s="4" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr"/>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>Edmondson, The Fearless Organization: Creating Psychological Safety in the Workplace for Learning, Innovation, and Growth (Wiley, 2018) — https://www.wiley.com/en-us/The+Fearless+Organization%3A+Creating+Psychological+Safety+in+the+Workplace+for+Learning%2C+Innovation%2C+and+Growth-p-9781119477242</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr"/>
+      <c r="D50" s="4" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr"/>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>Google re:Work, Guide: Understand Team Effectiveness (Project Aristotle research, accessed 2026-07) — https://rework.withgoogle.com/intl/en/guides/understand-team-effectiveness</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr"/>
+      <c r="D51" s="4" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr"/>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>Deci &amp; Ryan, The "What" and "Why" of Goal Pursuits: Human Needs and the Self-Determination of Behavior, Psychological Inquiry 11(4), 227-268 (2000) — https://doi.org/10.1207/S15327965PLI1104_01</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr"/>
+      <c r="D52" s="4" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr"/>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>Herzberg, One More Time: How Do You Motivate Employees?, Harvard Business Review 46(1), 53-62 (1968; HBR Classic reprint 2003) — https://hbr.org/2003/01/one-more-time-how-do-you-motivate-employees</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr"/>
+      <c r="D53" s="4" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr"/>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>Perri, Escaping the Build Trap: How Effective Product Management Creates Real Value (O'Reilly, 2018) — https://www.oreilly.com/library/view/escaping-the-build/9781491973783/</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr"/>
+      <c r="D54" s="4" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr"/>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>Skelton &amp; Pais, Team Topologies (IT Revolution, 2019)</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr"/>
+      <c r="D55" s="4" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr"/>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>Noda, Storey, Forsgren &amp; Greiler, DevEx: What Actually Drives Productivity, ACM Queue 21(2) (2023) — https://queue.acm.org/detail.cfm?id=3595878</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr"/>
+      <c r="D56" s="4" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr"/>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>Cagan, INSPIRED: How to Create Tech Products Customers Love, 2nd Edition (Wiley, 2018) — https://www.svpg.com/inspired-2nd-edition/</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr"/>
+      <c r="D57" s="4" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr"/>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>Spotify Engineering, How We Use Golden Paths to Solve Fragmentation in Our Software Ecosystem (Spotify Engineering Blog, 2020) — https://engineering.atspotify.com/2020/08/how-we-use-golden-paths-to-solve-fragmentation-in-our-software-ecosystem/</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr"/>
+      <c r="D58" s="4" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr"/>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>SFIA Foundation, Skills Framework for the Information Age, version 9 (2024) — https://sfia-online.org/en/sfia-9</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr"/>
+      <c r="D59" s="4" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr"/>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>Bottcher, What I Talk About When I Talk About Platforms (martinfowler.com, 2018) — https://martinfowler.com/articles/talk-about-platforms.html</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr"/>
+      <c r="D60" s="4" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr"/>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>Winters, Manshreck &amp; Wright, Software Engineering at Google: Lessons Learned from Programming Over Time (O'Reilly, 2020) — https://abseil.io/resources/swe-book</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr"/>
+      <c r="D61" s="4" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr"/>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>CNCF TAG App Delivery, Platform Engineering Maturity Model (2023) — https://tag-app-delivery.cncf.io/whitepapers/platform-eng-maturity-model/</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr"/>
+      <c r="D62" s="4" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr"/>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>Beyer, Jones, Petoff &amp; Murphy (eds.), Site Reliability Engineering: How Google Runs Production Systems (O'Reilly/Google, 2016) — https://sre.google/sre-book/table-of-contents/</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr"/>
+      <c r="D63" s="4" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr"/>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>PagerDuty, Incident Response Documentation (accessed 2026-07) — https://response.pagerduty.com/</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr"/>
+      <c r="D64" s="4" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr"/>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>Allspaw, Blameless PostMortems and a Just Culture, Code as Craft (Etsy Engineering Blog, 2012) — https://www.etsy.com/codeascraft/blameless-postmortems</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr"/>
+      <c r="D65" s="4" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr"/>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>Majors, Fong-Jones &amp; Miranda, Observability Engineering: Achieving Production Excellence (O'Reilly, 2022) — https://www.oreilly.com/library/view/observability-engineering/9781492076438/</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr"/>
+      <c r="D66" s="4" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr"/>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>Gregg, Systems Performance: Enterprise and the Cloud, 2nd ed. (Addison-Wesley, 2020) — https://www.brendangregg.com/systems-performance-2nd-edition-book.html</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr"/>
+      <c r="D67" s="4" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr"/>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>Conway, How Do Committees Invent?, Datamation 14(4), 28-31 (1968) — https://www.melconway.com/Home/Committees_Paper.html</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr"/>
+      <c r="D68" s="4" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr"/>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>Nygard, Documenting Architecture Decisions (Cognitect blog, 2011) — https://cognitect.com/blog/2011/11/15/documenting-architecture-decisions</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr"/>
+      <c r="D69" s="4" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr"/>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>Humble &amp; Farley, Continuous Delivery: Reliable Software Releases through Build Test and Deployment Automation (Addison-Wesley, 2010) — https://continuousdelivery.com/</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr"/>
+      <c r="D70" s="4" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="inlineStr"/>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>Cunningham, The WyCash Portfolio Management System, OOPSLA 1992 Experience Report — https://c2.com/doc/oopsla92.html</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr"/>
+      <c r="D71" s="4" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="inlineStr"/>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>Larson, An Elegant Puzzle: Systems of Engineering Management (Stripe Press, 2019) — https://press.stripe.com/an-elegant-puzzle</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr"/>
+      <c r="D72" s="4" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr"/>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>Wardley, Wardley Maps: Topographical Intelligence in Business (2016, online book) — https://wardleymaps.com/</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr"/>
+      <c r="D73" s="4" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="inlineStr"/>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t>Korn Ferry, Korn Ferry Leadership Architect Global Competency Framework (2014) — https://www.kornferry.com/capabilities/talent-suite/korn-ferry-assess/leadership-architect</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr"/>
+      <c r="D74" s="4" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr"/>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>OWASP Foundation, OWASP Application Security Verification Standard (accessed 2026-07) — https://owasp.org/www-project-application-security-verification-standard/</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr"/>
+      <c r="D75" s="4" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="inlineStr"/>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>McConnell, Software Estimation: Demystifying the Black Art (Microsoft Press, 2006) — https://www.construx.com/store/software-estimation-demystifying-the-black-art/</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr"/>
+      <c r="D76" s="4" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr"/>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>Reinertsen, The Principles of Product Development Flow: Second Generation Lean Product Development (Celeritas, 2009)</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr"/>
+      <c r="D77" s="4" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr"/>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>Brooks, The Mythical Man-Month: Essays on Software Engineering, Anniversary ed. (Addison-Wesley, 1995; orig. 1975) — https://en.wikipedia.org/wiki/The_Mythical_Man-Month</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr"/>
+      <c r="D78" s="4" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr"/>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>Forsgren, Humble &amp; Kim, Accelerate: The Science of Lean Software and DevOps (IT Revolution Press, 2018) — https://itrevolution.com/product/accelerate/</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr"/>
+      <c r="D79" s="4" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr"/>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>Forsgren, Storey, Maddila, Zimmermann, Houck &amp; Butler, The SPACE of Developer Productivity, ACM Queue 19(1) (2021) — https://queue.acm.org/detail.cfm?id=3454124</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr"/>
+      <c r="D80" s="4" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr"/>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>Deming, Out of the Crisis (MIT Center for Advanced Engineering Study, 1986)</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr"/>
+      <c r="D81" s="4" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="inlineStr"/>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>NIST, The NIST Cybersecurity Framework (CSF) 2.0, NIST CSWP 29 (2024) — https://csrc.nist.gov/pubs/cswp/29/the-nist-cybersecurity-framework-csf-20/final</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="inlineStr"/>
+      <c r="D82" s="4" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr"/>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>Project Management Institute, A Guide to the Project Management Body of Knowledge (PMBOK Guide), 7th ed. (PMI, 2021) — https://www.pmi.org/standards/pmbok</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr"/>
+      <c r="D83" s="4" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr"/>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>Rumelt, Good Strategy Bad Strategy: The Difference and Why It Matters (Crown Business, 2011) — https://www.penguinrandomhouse.com/books/198888/good-strategy-bad-strategy-by-richard-p-rumelt/</t>
+        </is>
+      </c>
+      <c r="C84" s="4" t="inlineStr"/>
+      <c r="D84" s="4" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr"/>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>Kotter, Leading Change (Harvard Business School Press, 1996) — https://openlibrary.org/books/OL982607M/Leading_Change</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr"/>
+      <c r="D85" s="4" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr"/>
+      <c r="B86" s="4" t="inlineStr">
+        <is>
+          <t>Duarte, HBR Guide to Persuasive Presentations (Harvard Business Review Press, 2012) — https://store.hbr.org/product/hbr-guide-to-persuasive-presentations/10058</t>
+        </is>
+      </c>
+      <c r="C86" s="4" t="inlineStr"/>
+      <c r="D86" s="4" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="inlineStr"/>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>Freeman, Strategic Management: A Stakeholder Approach (Pitman, 1984)</t>
+        </is>
+      </c>
+      <c r="C87" s="4" t="inlineStr"/>
+      <c r="D87" s="4" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="4" t="inlineStr"/>
+      <c r="B88" s="4" t="inlineStr">
+        <is>
+          <t>Cohen &amp; Bradford, Influence Without Authority, 3rd ed. (Wiley, 2017) — https://www.wiley.com/en-us/Influence+Without+Authority,+3rd+Edition-p-9781119347712</t>
+        </is>
+      </c>
+      <c r="C88" s="4" t="inlineStr"/>
+      <c r="D88" s="4" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="4" t="inlineStr"/>
+      <c r="B89" s="4" t="inlineStr">
+        <is>
+          <t>Bungay, The Art of Action: How Leaders Close the Gaps between Plans, Actions and Results (Nicholas Brealey, 2011)</t>
+        </is>
+      </c>
+      <c r="C89" s="4" t="inlineStr"/>
+      <c r="D89" s="4" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="4" t="inlineStr"/>
+      <c r="B90" s="4" t="inlineStr">
+        <is>
+          <t>Drucker, The Effective Executive (Harper &amp; Row, 1967)</t>
+        </is>
+      </c>
+      <c r="C90" s="4" t="inlineStr"/>
+      <c r="D90" s="4" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="inlineStr"/>
+      <c r="B91" s="4" t="inlineStr">
+        <is>
+          <t>Marquet, Turn the Ship Around!: A True Story of Turning Followers into Leaders (Portfolio/Penguin, 2013; orig. 2012)</t>
+        </is>
+      </c>
+      <c r="C91" s="4" t="inlineStr"/>
+      <c r="D91" s="4" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="4" t="inlineStr"/>
+      <c r="B92" s="4" t="inlineStr">
+        <is>
+          <t>Eurich, What Self-Awareness Really Is (and How to Cultivate It), Harvard Business Review (2018) — https://hbr.org/2018/01/what-self-awareness-really-is-and-how-to-cultivate-it</t>
+        </is>
+      </c>
+      <c r="C92" s="4" t="inlineStr"/>
+      <c r="D92" s="4" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="4" t="inlineStr"/>
+      <c r="B93" s="4" t="inlineStr">
+        <is>
+          <t>Lombardo &amp; Eichinger, The Career Architect Development Planner, 3rd ed. (Lominger, 2000)</t>
+        </is>
+      </c>
+      <c r="C93" s="4" t="inlineStr"/>
+      <c r="D93" s="4" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="4" t="inlineStr"/>
+      <c r="B94" s="4" t="inlineStr">
+        <is>
+          <t>Loehr &amp; Schwartz, The Power of Full Engagement: Managing Energy, Not Time, Is the Key to High Performance and Personal Renewal (Free Press, 2003)</t>
+        </is>
+      </c>
+      <c r="C94" s="4" t="inlineStr"/>
+      <c r="D94" s="4" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="4" t="inlineStr"/>
+      <c r="B95" s="4" t="inlineStr">
+        <is>
+          <t>Kahneman, Thinking, Fast and Slow (Farrar, Straus and Giroux, 2011) — https://en.wikipedia.org/wiki/Thinking,_Fast_and_Slow</t>
+        </is>
+      </c>
+      <c r="C95" s="4" t="inlineStr"/>
+      <c r="D95" s="4" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="4" t="inlineStr"/>
+      <c r="B96" s="4" t="inlineStr">
+        <is>
+          <t>Mayer, Davis &amp; Schoorman, An Integrative Model of Organizational Trust, Academy of Management Review 20(3), 709-734 (1995) — https://people.wku.edu/richard.miller/Mayer%20Trust%20article.pdf</t>
+        </is>
+      </c>
+      <c r="C96" s="4" t="inlineStr"/>
+      <c r="D96" s="4" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="4" t="inlineStr"/>
+      <c r="B97" s="4" t="inlineStr">
+        <is>
+          <t>ACM, ACM Code of Ethics and Professional Conduct (2018) — https://www.acm.org/code-of-ethics</t>
+        </is>
+      </c>
+      <c r="C97" s="4" t="inlineStr"/>
+      <c r="D97" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>